<commit_message>
feat: add teacher and staff management modules
- Implement Firestore CRUD for teacher and admin records
- Add TeacherFormScreen component for data entry
- Introduce global error suppression for app stability
- Enhance clipboard interaction and toast notifications
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -14809,7 +14809,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -14848,581 +14848,12 @@
         <v>ملاحظات</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>30</v>
-      </c>
-      <c r="B3" t="str">
-        <v>ابو السعود معاوية ابو السعود</v>
-      </c>
-      <c r="C3" t="str">
-        <v>حارس</v>
-      </c>
-      <c r="D3" t="str">
-        <v>متوسط وثانوي</v>
-      </c>
-      <c r="E3" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2474277379</v>
-      </c>
-      <c r="G3" t="str">
-        <v>السودان</v>
-      </c>
-      <c r="H3" t="str">
-        <v>0554292056</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>295</v>
-      </c>
-      <c r="B4" t="str">
-        <v>صبري محمد محمود عثمان</v>
-      </c>
-      <c r="C4" t="str">
-        <v>حارس</v>
-      </c>
-      <c r="D4" t="str">
-        <v>ثانوي بنين</v>
-      </c>
-      <c r="E4" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F4" t="str">
-        <v>2207392172</v>
-      </c>
-      <c r="H4" t="str">
-        <v>553833279</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>293</v>
-      </c>
-      <c r="B5" t="str">
-        <v>عاطف محمد ادريس محمد</v>
-      </c>
-      <c r="C5" t="str">
-        <v>حارس</v>
-      </c>
-      <c r="D5" t="str">
-        <v>أقسام البنين</v>
-      </c>
-      <c r="E5" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F5" t="str">
-        <v>2276755655</v>
-      </c>
-      <c r="G5" t="str">
-        <v>السودان</v>
-      </c>
-      <c r="H5" t="str">
-        <v>552178464</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>3028</v>
-      </c>
-      <c r="B6" t="str">
-        <v>ابوبكر صديق</v>
-      </c>
-      <c r="C6" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D6" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E6" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2539904892</v>
-      </c>
-      <c r="G6" t="str">
-        <v>بنجلاديش</v>
-      </c>
-      <c r="H6" t="str">
-        <v>0571650836</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>324</v>
-      </c>
-      <c r="B7" t="str">
-        <v>صابير جولا</v>
-      </c>
-      <c r="C7" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D7" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E7" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F7">
-        <v>2429034354</v>
-      </c>
-      <c r="G7" t="str">
-        <v>نيبالي</v>
-      </c>
-      <c r="H7" t="str">
-        <v>500798824</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>3442</v>
-      </c>
-      <c r="B8" t="str">
-        <v>فيضان احمد</v>
-      </c>
-      <c r="C8" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D8" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E8" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2555671813</v>
-      </c>
-      <c r="G8" t="str">
-        <v>الهند</v>
-      </c>
-      <c r="H8" t="str">
-        <v>0575249055</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>3441</v>
-      </c>
-      <c r="B9" t="str">
-        <v>محمد علي</v>
-      </c>
-      <c r="C9" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D9" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E9" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F9" t="str">
-        <v>2555671722</v>
-      </c>
-      <c r="G9" t="str">
-        <v>الهند</v>
-      </c>
-      <c r="H9" t="str">
-        <v>0571187133</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>319</v>
-      </c>
-      <c r="B10" t="str">
-        <v>نجم الدين خان</v>
-      </c>
-      <c r="C10" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D10" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E10" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F10" t="str">
-        <v>2429347194</v>
-      </c>
-      <c r="G10" t="str">
-        <v>نيبالي</v>
-      </c>
-      <c r="H10" t="str">
-        <v>0576104814</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>4625</v>
-      </c>
-      <c r="B11" t="str">
-        <v>نادر محمد عبد الهادي</v>
-      </c>
-      <c r="C11" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D11" t="str">
-        <v>الابتدائي والمتوسط</v>
-      </c>
-      <c r="E11" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F11" t="str">
-        <v>2615293293</v>
-      </c>
-      <c r="G11" t="str">
-        <v>مصر</v>
-      </c>
-      <c r="H11" t="str">
-        <v>0544388592</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="str">
-        <v>عتيق آل رامان</v>
-      </c>
-      <c r="C12" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="D12" t="str">
-        <v>كل المراحل</v>
-      </c>
-      <c r="E12" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F12" t="str">
-        <v>2552787216</v>
-      </c>
-      <c r="G12" t="str">
-        <v>الهند</v>
-      </c>
-      <c r="H12" t="str">
-        <v>0572188404</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>322</v>
-      </c>
-      <c r="B13" t="str">
-        <v>رانجيت مهاسيز</v>
-      </c>
-      <c r="C13" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="D13" t="str">
-        <v>الثانوية</v>
-      </c>
-      <c r="E13" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F13" t="str">
-        <v>2428894089</v>
-      </c>
-      <c r="G13" t="str">
-        <v>نيبالي</v>
-      </c>
-      <c r="H13" t="str">
-        <v>0557887356</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>315</v>
-      </c>
-      <c r="B14" t="str">
-        <v>شهيد الإسلام أنو مياه</v>
-      </c>
-      <c r="C14" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="D14" t="str">
-        <v>الابتدائية</v>
-      </c>
-      <c r="E14" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F14" t="str">
-        <v>2268093669</v>
-      </c>
-      <c r="G14" t="str">
-        <v>بنجلاديش</v>
-      </c>
-      <c r="H14" t="str">
-        <v>530195994</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>321</v>
-      </c>
-      <c r="B15" t="str">
-        <v>بابلو مهاسيز</v>
-      </c>
-      <c r="C15" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="D15" t="str">
-        <v>الابتدائية</v>
-      </c>
-      <c r="E15" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F15" t="str">
-        <v>2428894311</v>
-      </c>
-      <c r="G15" t="str">
-        <v>نيبالي</v>
-      </c>
-      <c r="H15" t="str">
-        <v>0572556532</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>328</v>
-      </c>
-      <c r="B16" t="str">
-        <v>نور الحق اكي اولادير</v>
-      </c>
-      <c r="C16" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="D16" t="str">
-        <v>الثانوية</v>
-      </c>
-      <c r="E16" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F16" t="str">
-        <v>2432179014</v>
-      </c>
-      <c r="G16" t="str">
-        <v>بنجلاديش</v>
-      </c>
-      <c r="H16" t="str">
-        <v>572293461</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>329</v>
-      </c>
-      <c r="B17" t="str">
-        <v>جيرالد اوغستين</v>
-      </c>
-      <c r="C17" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="D17" t="str">
-        <v>إدارة المجمع</v>
-      </c>
-      <c r="E17" t="str">
-        <v xml:space="preserve">بنين </v>
-      </c>
-      <c r="F17" t="str">
-        <v>2443914516</v>
-      </c>
-      <c r="G17" t="str">
-        <v>الفلبين</v>
-      </c>
-      <c r="H17" t="str">
-        <v>573082979</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>341</v>
-      </c>
-      <c r="B18" t="str">
-        <v>لوسيلا نينادا كابانيرو</v>
-      </c>
-      <c r="C18" t="str">
-        <v>عاملة نظافة</v>
-      </c>
-      <c r="D18" t="str">
-        <v>الثانوية</v>
-      </c>
-      <c r="E18" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F18" t="str">
-        <v>2444621433</v>
-      </c>
-      <c r="G18" t="str">
-        <v>الفلبين</v>
-      </c>
-      <c r="H18" t="str">
-        <v>503306948</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>344</v>
-      </c>
-      <c r="B19" t="str">
-        <v>ميشيل كالدو توبالاس</v>
-      </c>
-      <c r="C19" t="str">
-        <v>عاملة نظافة</v>
-      </c>
-      <c r="D19" t="str">
-        <v>التمهيدية</v>
-      </c>
-      <c r="E19" t="str">
-        <v>بنات</v>
-      </c>
-      <c r="F19" t="str">
-        <v>2442596603</v>
-      </c>
-      <c r="G19" t="str">
-        <v>الفلبين</v>
-      </c>
-      <c r="H19" t="str">
-        <v>570456403</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" t="str">
-        <v>الوظيفة / المرحلة</v>
-      </c>
-      <c r="C21" t="str">
-        <v>تمهيدي</v>
-      </c>
-      <c r="D21" t="str">
-        <v>ابتدائي بنات</v>
-      </c>
-      <c r="E21" t="str">
-        <v>ابتدائي بنين</v>
-      </c>
-      <c r="F21" t="str">
-        <v>متوسط بنات</v>
-      </c>
-      <c r="G21" t="str">
-        <v>ثانوي بنين</v>
-      </c>
-      <c r="H21" t="str">
-        <v>ثانوي بنات</v>
-      </c>
-      <c r="I21" t="str">
-        <v>ادارة المجمع</v>
-      </c>
-      <c r="J21" t="str">
-        <v>الاجمالي</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" t="str">
-        <v>عامل نظافة</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="E22">
-        <v>2</v>
-      </c>
-      <c r="G22">
-        <v>2</v>
-      </c>
-      <c r="H22">
-        <v>1</v>
-      </c>
-      <c r="I22">
-        <v>1</v>
-      </c>
-      <c r="J22">
-        <f>SUM(C22:I22)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" t="str">
-        <v>حارس</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>1</v>
-      </c>
-      <c r="H23">
-        <v>1</v>
-      </c>
-      <c r="J23">
-        <f>SUM(C23:I23)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" t="str">
-        <v>سائق</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="H24">
-        <v>2</v>
-      </c>
-      <c r="J24">
-        <f>SUM(C24:I24)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" t="str">
-        <v>إجمالي الخدمات المساندة أفراد</v>
-      </c>
-      <c r="C25">
-        <f>SUM(C22:C24)</f>
-        <v>2</v>
-      </c>
-      <c r="D25">
-        <f>SUM(D22:D24)</f>
-        <v>2</v>
-      </c>
-      <c r="E25">
-        <f>SUM(E22:E24)</f>
-        <v>4</v>
-      </c>
-      <c r="F25">
-        <f>SUM(F22:F24)</f>
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <f>SUM(G22:G24)</f>
-        <v>3</v>
-      </c>
-      <c r="H25">
-        <f>SUM(H22:H24)</f>
-        <v>4</v>
-      </c>
-      <c r="I25">
-        <f>SUM(I22:I24)</f>
-        <v>1</v>
-      </c>
-      <c r="J25">
-        <f>SUM(C25:I25)</f>
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <pageMargins left="0.15748031496062992" right="0.15748031496062992" top="0.4330708661417323" bottom="0.2" header="0.31496062992125984" footer="0.17"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add mapping for flexible assignment sheet names
Implement automatic sheet name resolution between "الاسنادات" and "اسناد بنين ف١" and ensure data merging for "اسناد البنات ف١" to improve data consistency when loading assignment files.
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -26,6 +26,7 @@
     <sheet name="القدرات والتحصيلي" sheetId="21" r:id="rId21"/>
     <sheet name="تصنيف العاملين " sheetId="22" r:id="rId22"/>
     <sheet name="العهدة المالية" sheetId="23" r:id="rId23"/>
+    <sheet name="الاسنادات" sheetId="24" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'إحصاء التخصصات'!#REF!</definedName>
@@ -12009,14 +12010,14 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E133"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v/>
       </c>
       <c r="B1" t="str">
-        <v/>
+        <v>اسنادات قطاع البنين</v>
       </c>
       <c r="C1" t="str">
         <v/>
@@ -12033,7 +12034,7 @@
         <v/>
       </c>
       <c r="B2" t="str">
-        <v>اسنادات ابتدائي</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -12064,67 +12065,67 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>المعلم</v>
+        <v/>
       </c>
       <c r="B4" t="str">
-        <v>المادة</v>
+        <v>اسنادات ابتدائي (بنين)</v>
       </c>
       <c r="C4" t="str">
-        <v>عدد حصص المعلم بالمدرسة</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>الإسناد</v>
+        <v/>
       </c>
       <c r="E4" t="str">
-        <v>إجمالي نصاب المعلم</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>العفيفي عبد الجواد</v>
+        <v/>
       </c>
       <c r="B5" t="str">
-        <v>معلم صف أول</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>24</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>24</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>محمود عبدالحسيب</v>
+        <v>المعلم</v>
       </c>
       <c r="B6" t="str">
-        <v>معلم صف أول</v>
+        <v>المادة</v>
       </c>
       <c r="C6" t="str">
-        <v>24</v>
+        <v>عدد حصص المعلم بالمدرسة</v>
       </c>
       <c r="D6" t="str">
-        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
+        <v>الإسناد</v>
       </c>
       <c r="E6" t="str">
-        <v>24</v>
+        <v>إجمالي نصاب المعلم</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>عبد العزيز يونس</v>
+        <v>العفيفي عبد الجواد</v>
       </c>
       <c r="B7" t="str">
-        <v>معلم صف ثاني</v>
+        <v>معلم صف أول</v>
       </c>
       <c r="C7" t="str">
         <v>24</v>
       </c>
       <c r="D7" t="str">
-        <v xml:space="preserve">(١٤) لغتي ص٢ فصلين + (١٠) اسلاميات ص٢ فصلين </v>
+        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
       </c>
       <c r="E7" t="str">
         <v>24</v>
@@ -12132,16 +12133,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>حسن عزالدين مبروك</v>
+        <v>محمود عبدالحسيب</v>
       </c>
       <c r="B8" t="str">
-        <v>معلم صف ثالث</v>
+        <v>معلم صف أول</v>
       </c>
       <c r="C8" t="str">
         <v>24</v>
       </c>
       <c r="D8" t="str">
-        <v>(١٤) لغتي ص٣ فصلين(2/4 ، 3/4) + (١٠) اسلاميات ص٣ فصلين +(٢) مهارات حياتية ص٣ فصلين</v>
+        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
       </c>
       <c r="E8" t="str">
         <v>24</v>
@@ -12149,16 +12150,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>سلمان حمد الفراج</v>
+        <v>عبد العزيز يونس</v>
       </c>
       <c r="B9" t="str">
-        <v>اسلاميات</v>
+        <v>معلم صف ثاني</v>
       </c>
       <c r="C9" t="str">
         <v>24</v>
       </c>
       <c r="D9" t="str">
-        <v>(١٢) اسلاميات ص٤ فصلين (2/4 ،3/4)+ (٨) اسلاميات ص٥+ (٤) اسلاميات ص٦ فصلين</v>
+        <v xml:space="preserve">(١٤) لغتي ص٢ فصلين + (١٠) اسلاميات ص٢ فصلين </v>
       </c>
       <c r="E9" t="str">
         <v>24</v>
@@ -12166,33 +12167,33 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>محمد الغباشي</v>
+        <v>حسن عزالدين مبروك</v>
       </c>
       <c r="B10" t="str">
-        <v>لغة عربية</v>
+        <v>معلم صف ثالث</v>
       </c>
       <c r="C10" t="str">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" t="str">
-        <v>(٥) لغتي ص 4 فصل(2/4) + (١٠) لغتي ص٥ فصلين +(١٠) لغتي ص٦ فصلين</v>
+        <v>(١٤) لغتي ص٣ فصلين(2/4 ، 3/4) + (١٠) اسلاميات ص٣ فصلين +(٢) مهارات حياتية ص٣ فصلين</v>
       </c>
       <c r="E10" t="str">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>طارق عبدالظاهر</v>
+        <v>سلمان حمد الفراج</v>
       </c>
       <c r="B11" t="str">
-        <v>رياضيات</v>
+        <v>اسلاميات</v>
       </c>
       <c r="C11" t="str">
         <v>24</v>
       </c>
       <c r="D11" t="str">
-        <v>(18) رياضيات ص٤ +(6) رياضيات ص٥ فصل</v>
+        <v>(١٢) اسلاميات ص٤ فصلين (2/4 ،3/4)+ (٨) اسلاميات ص٥+ (٤) اسلاميات ص٦ فصلين</v>
       </c>
       <c r="E11" t="str">
         <v>24</v>
@@ -12200,24 +12201,24 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">احمد سالم </v>
+        <v>محمد الغباشي</v>
       </c>
       <c r="B12" t="str">
-        <v>رياضيات</v>
+        <v>لغة عربية</v>
       </c>
       <c r="C12" t="str">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" t="str">
-        <v>(١٢) رياضيات ص٦ فصلين  + مسند (6) رياضيات ص5 فصل + (5) نشاط ص4 وص5 + (1) نشاط ص6 فصل</v>
+        <v>(٥) لغتي ص 4 فصل(2/4) + (١٠) لغتي ص٥ فصلين +(١٠) لغتي ص٦ فصلين</v>
       </c>
       <c r="E12" t="str">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">عمرو محمد </v>
+        <v>طارق عبدالظاهر</v>
       </c>
       <c r="B13" t="str">
         <v>رياضيات</v>
@@ -12226,7 +12227,7 @@
         <v>24</v>
       </c>
       <c r="D13" t="str">
-        <v xml:space="preserve">(12) رياضيات ص٢ ب فصلين+(12) رياضيات ص٣ فصلين </v>
+        <v>(18) رياضيات ص٤ +(6) رياضيات ص٥ فصل</v>
       </c>
       <c r="E13" t="str">
         <v>24</v>
@@ -12234,16 +12235,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ربيع عوض</v>
+        <v xml:space="preserve">احمد سالم </v>
       </c>
       <c r="B14" t="str">
-        <v>لغة انجليزية</v>
+        <v>رياضيات</v>
       </c>
       <c r="C14" t="str">
         <v>24</v>
       </c>
       <c r="D14" t="str">
-        <v>(٦) E ص٥ + (٦) E ص٦ + (٩) E ص٤ + (2) انجليزي إثرائي ص6 + (1) نشاط ص6 فصل</v>
+        <v>(١٢) رياضيات ص٦ فصلين  + مسند (6) رياضيات ص5 فصل + (5) نشاط ص4 وص5 + (1) نشاط ص6 فصل</v>
       </c>
       <c r="E14" t="str">
         <v>24</v>
@@ -12251,16 +12252,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>محمد السيد</v>
+        <v xml:space="preserve">عمرو محمد </v>
       </c>
       <c r="B15" t="str">
-        <v>لغة انجليزية</v>
+        <v>رياضيات</v>
       </c>
       <c r="C15" t="str">
         <v>24</v>
       </c>
       <c r="D15" t="str">
-        <v xml:space="preserve"> (٦) E ص٣ + + (٤) E اثرائي ص3  + (٦) E اثرائي ص٤ + (2) E اثرائي ص٦+ (٤) E اثراىي ص٥ +(2) انجليزي اثرائي ص2 فصل</v>
+        <v xml:space="preserve">(12) رياضيات ص٢ ب فصلين+(12) رياضيات ص٣ فصلين </v>
       </c>
       <c r="E15" t="str">
         <v>24</v>
@@ -12268,7 +12269,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>احمد حسنين</v>
+        <v>ربيع عوض</v>
       </c>
       <c r="B16" t="str">
         <v>لغة انجليزية</v>
@@ -12277,7 +12278,7 @@
         <v>24</v>
       </c>
       <c r="D16" t="str">
-        <v>(6) E ص١+ (٤) E اثرائي ص١+ (٦) E ص٢ + (2) E اثرائي ص٢ فصل+ (4) ماث ص١ + (٢) ساينس ص١</v>
+        <v>(٦) E ص٥ + (٦) E ص٦ + (٩) E ص٤ + (2) انجليزي إثرائي ص6 + (1) نشاط ص6 فصل</v>
       </c>
       <c r="E16" t="str">
         <v>24</v>
@@ -12285,16 +12286,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve"> ايمن محمد </v>
+        <v>محمد السيد</v>
       </c>
       <c r="B17" t="str">
-        <v>علوم</v>
+        <v>لغة انجليزية</v>
       </c>
       <c r="C17" t="str">
         <v>24</v>
       </c>
       <c r="D17" t="str">
-        <v>(٦) علوم ص2 فصلين+ (8) علوم ص٣ فصلين+ (٨) علوم ص4 فصلين(1/4،2/4)+ (٢) بدنية ص5 فصل (2/5)</v>
+        <v xml:space="preserve"> (٦) E ص٣ + + (٤) E اثرائي ص3  + (٦) E اثرائي ص٤ + (2) E اثرائي ص٦+ (٤) E اثراىي ص٥ +(2) انجليزي اثرائي ص2 فصل</v>
       </c>
       <c r="E17" t="str">
         <v>24</v>
@@ -12302,16 +12303,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>مصطفى عبدالتواب</v>
+        <v>احمد حسنين</v>
       </c>
       <c r="B18" t="str">
-        <v>علوم</v>
+        <v>لغة انجليزية</v>
       </c>
       <c r="C18" t="str">
         <v>24</v>
       </c>
       <c r="D18" t="str">
-        <v>(٨) علوم ص٥  + (٨) علوم ص٦ + (٤) علوم ص٤ + (٤) اجتماعيات ص٦</v>
+        <v>(6) E ص١+ (٤) E اثرائي ص١+ (٦) E ص٢ + (2) E اثرائي ص٢ فصل+ (4) ماث ص١ + (٢) ساينس ص١</v>
       </c>
       <c r="E18" t="str">
         <v>24</v>
@@ -12319,16 +12320,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>محمد إبراهيم</v>
+        <v xml:space="preserve"> ايمن محمد </v>
       </c>
       <c r="B19" t="str">
-        <v>لغة عربية</v>
+        <v>علوم</v>
       </c>
       <c r="C19" t="str">
         <v>24</v>
       </c>
       <c r="D19" t="str">
-        <v>(١٠) لغتي ص٤ فصلين(1/4،3/4) + (٤) اسلاميات ص4 فصل(1/4) + (١٠) اجتماعيات ص٤ فصلين ص٥ فصلين</v>
+        <v>(٦) علوم ص2 فصلين+ (8) علوم ص٣ فصلين+ (٨) علوم ص4 فصلين(1/4،2/4)+ (٢) بدنية ص5 فصل (2/5)</v>
       </c>
       <c r="E19" t="str">
         <v>24</v>
@@ -12336,16 +12337,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>رامي يسن معروف</v>
+        <v>مصطفى عبدالتواب</v>
       </c>
       <c r="B20" t="str">
-        <v>فنية</v>
+        <v>علوم</v>
       </c>
       <c r="C20" t="str">
         <v>24</v>
       </c>
       <c r="D20" t="str">
-        <v>(٤) فنية ص٢+ (٤) فنية ص٣ + (٣) فنية ص٤ + (٢) فنية ص٥ + (٢) فنية ص٦ + (٩) مهارات حياتية ص٢، ص٤، ص٥، ص٦</v>
+        <v>(٨) علوم ص٥  + (٨) علوم ص٦ + (٤) علوم ص٤ + (٤) اجتماعيات ص٦</v>
       </c>
       <c r="E20" t="str">
         <v>24</v>
@@ -12353,16 +12354,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>محمود وحش</v>
+        <v>محمد إبراهيم</v>
       </c>
       <c r="B21" t="str">
-        <v>بدنية</v>
+        <v>لغة عربية</v>
       </c>
       <c r="C21" t="str">
         <v>24</v>
       </c>
       <c r="D21" t="str">
-        <v>(6) بدنية ص٣ + (٦) بدنية ص٤ + (6) بدنية ص٢  + (2) بدنية ص٥ +  (4) بدنية ص6</v>
+        <v>(١٠) لغتي ص٤ فصلين(1/4،3/4) + (٤) اسلاميات ص4 فصل(1/4) + (١٠) اجتماعيات ص٤ فصلين ص٥ فصلين</v>
       </c>
       <c r="E21" t="str">
         <v>24</v>
@@ -12370,32 +12371,66 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>آمير جلال</v>
+        <v>رامي يسن معروف</v>
       </c>
       <c r="B22" t="str">
-        <v>رقمية</v>
+        <v>فنية</v>
       </c>
       <c r="C22" t="str">
         <v>24</v>
       </c>
       <c r="D22" t="str">
-        <v xml:space="preserve">(2) رقمية ص١+ (٤) رقمية ص٢+ (٤) رقمية ص٣ + (٦) رقمية ص٤ + (٤) رقمية ص٥ + (٤) رقمية ص٦ </v>
+        <v>(٤) فنية ص٢+ (٤) فنية ص٣ + (٣) فنية ص٤ + (٢) فنية ص٥ + (٢) فنية ص٦ + (٩) مهارات حياتية ص٢، ص٤، ص٥، ص٦</v>
       </c>
       <c r="E22" t="str">
         <v>24</v>
       </c>
     </row>
-    <row r="23" xml:space="preserve">
+    <row r="23">
       <c r="A23" t="str">
+        <v>محمود وحش</v>
+      </c>
+      <c r="B23" t="str">
+        <v>بدنية</v>
+      </c>
+      <c r="C23" t="str">
+        <v>24</v>
+      </c>
+      <c r="D23" t="str">
+        <v>(6) بدنية ص٣ + (٦) بدنية ص٤ + (6) بدنية ص٢  + (2) بدنية ص٥ +  (4) بدنية ص6</v>
+      </c>
+      <c r="E23" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>آمير جلال</v>
+      </c>
+      <c r="B24" t="str">
+        <v>رقمية</v>
+      </c>
+      <c r="C24" t="str">
+        <v>24</v>
+      </c>
+      <c r="D24" t="str">
+        <v xml:space="preserve">(2) رقمية ص١+ (٤) رقمية ص٢+ (٤) رقمية ص٣ + (٦) رقمية ص٤ + (٤) رقمية ص٥ + (٤) رقمية ص٦ </v>
+      </c>
+      <c r="E24" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
         <v>إجمالي الحصص</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B25" t="str">
         <v>396</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C25" t="str">
         <v>433</v>
       </c>
-      <c r="D23" t="str" xml:space="preserve">
+      <c r="D25" t="str" xml:space="preserve">
         <v xml:space="preserve">اضافة عدد (٣٨) حصة اثرائي لغة انجليزية + (١٢) اثرائي رقمية صفوف أولية فيصبح مجموع الحصص الاثرائية (٥٠) حصة _x000d_
 تخفيض (١) حصة فنية الصف الاول باجمالي (٢) حصة_x000d_
 تخفيض (١) حصة بدنية الصف الاول باجمالي (٢) حصة_x000d_
@@ -12405,40 +12440,6 @@
 استبدال  (٣٢) حصة نشاط  مع الحصص الاثرائية _x000d_
 (٥٠) - (٣٢) = (١٨) حصة </v>
       </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v/>
-      </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
-      <c r="E24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>اسنادات متوسط دار القلم الفصل الاول 1447</v>
-      </c>
-      <c r="B25" t="str">
-        <v/>
-      </c>
-      <c r="C25" t="str">
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
       <c r="E25" t="str">
         <v/>
       </c>
@@ -12462,135 +12463,135 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>المعلم</v>
+        <v/>
       </c>
       <c r="B27" t="str">
-        <v>المادة</v>
+        <v>اسنادات متوسط (بنين)</v>
       </c>
       <c r="C27" t="str">
-        <v>عدد حصص المعلم بالمدرسة</v>
+        <v/>
       </c>
       <c r="D27" t="str">
-        <v>الإسناد</v>
+        <v/>
       </c>
       <c r="E27" t="str">
-        <v>إجمالي نصاب المعلم</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>فواز المطيري</v>
+        <v/>
       </c>
       <c r="B28" t="str">
-        <v>اسلاميات</v>
+        <v/>
       </c>
       <c r="C28" t="str">
-        <v>25</v>
+        <v/>
       </c>
       <c r="D28" t="str">
-        <v xml:space="preserve"> (5) اسلاميات ص1 فصل 1/1 +(10) اسلاميات ص2 فصلين 2/1 - 2/2 + (10) اسلاميات ص 3 فصل 3/1 - 3/2 </v>
+        <v/>
       </c>
       <c r="E28" t="str">
-        <v>25</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>احمد صوفي</v>
+        <v>المعلم</v>
       </c>
       <c r="B29" t="str">
-        <v>لغة عربية</v>
+        <v>المادة</v>
       </c>
       <c r="C29" t="str">
-        <v>26</v>
+        <v>عدد حصص المعلم بالمدرسة</v>
       </c>
       <c r="D29" t="str">
-        <v xml:space="preserve"> (15) لغتي ص1 متوسط   +  (٥) اسلاميات ص2  فصل 2/3  +(6) تفكير ناقد متوسط ص٣</v>
+        <v>الإسناد</v>
       </c>
       <c r="E29" t="str">
-        <v>26</v>
+        <v>إجمالي نصاب المعلم</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>محمد سمير</v>
+        <v>فواز المطيري</v>
       </c>
       <c r="B30" t="str">
-        <v>لغة عربية</v>
+        <v>اسلاميات</v>
       </c>
       <c r="C30" t="str">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D30" t="str">
-        <v xml:space="preserve">(15) لغتي ص2 م + (12 ) لغتي ص 3 </v>
+        <v xml:space="preserve"> (5) اسلاميات ص1 فصل 1/1 +(10) اسلاميات ص2 فصلين 2/1 - 2/2 + (10) اسلاميات ص 3 فصل 3/1 - 3/2 </v>
       </c>
       <c r="E30" t="str">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ماهر الحربي</v>
+        <v>احمد صوفي</v>
       </c>
       <c r="B31" t="str">
-        <v>رياضيات</v>
+        <v>لغة عربية</v>
       </c>
       <c r="C31" t="str">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D31" t="str">
-        <v>(18) رياضيات ص١+ (6) رياضيات ص2م فصل 2/3</v>
+        <v xml:space="preserve"> (15) لغتي ص1 متوسط   +  (٥) اسلاميات ص2  فصل 2/3  +(6) تفكير ناقد متوسط ص٣</v>
       </c>
       <c r="E31" t="str">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>حسن السيد</v>
+        <v>محمد سمير</v>
       </c>
       <c r="B32" t="str">
-        <v>رياضيات</v>
+        <v>لغة عربية</v>
       </c>
       <c r="C32" t="str">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D32" t="str">
-        <v>(18) رياضيات ص3م  + (6) رياضيات ص2م فصل 2/2 - 2/3</v>
+        <v xml:space="preserve">(15) لغتي ص2 م + (12 ) لغتي ص 3 </v>
       </c>
       <c r="E32" t="str">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">سلمان الصادق </v>
+        <v>ماهر الحربي</v>
       </c>
       <c r="B33" t="str">
-        <v>لغة انجليزية</v>
+        <v>رياضيات</v>
       </c>
       <c r="C33" t="str">
         <v>24</v>
       </c>
       <c r="D33" t="str">
-        <v xml:space="preserve">(12) انجليزي ص٢متوسط +(12) انجليزي ص٣ متوسط  </v>
+        <v>(18) رياضيات ص١+ (6) رياضيات ص2م فصل 2/3</v>
       </c>
       <c r="E33" t="str">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>مصطفى فتحي</v>
+        <v>حسن السيد</v>
       </c>
       <c r="B34" t="str">
-        <v>لغة انجليزية</v>
+        <v>رياضيات</v>
       </c>
       <c r="C34" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D34" t="str">
-        <v xml:space="preserve"> (١٢) انجليزي ص١ متوسط + مكمل (١٢) حصة بالثانوي </v>
+        <v>(18) رياضيات ص3م  + (6) رياضيات ص2م فصل 2/2 - 2/3</v>
       </c>
       <c r="E34" t="str">
         <v>24</v>
@@ -12598,16 +12599,16 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>فارس الجندي</v>
+        <v xml:space="preserve">سلمان الصادق </v>
       </c>
       <c r="B35" t="str">
-        <v>علوم</v>
+        <v>لغة انجليزية</v>
       </c>
       <c r="C35" t="str">
         <v>24</v>
       </c>
       <c r="D35" t="str">
-        <v xml:space="preserve">(12) علوم ص١ +(12) علوم ص٢ </v>
+        <v xml:space="preserve">(12) انجليزي ص٢متوسط +(12) انجليزي ص٣ متوسط  </v>
       </c>
       <c r="E35" t="str">
         <v>24</v>
@@ -12615,33 +12616,33 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">محمد العشماوي </v>
+        <v>مصطفى فتحي</v>
       </c>
       <c r="B36" t="str">
-        <v>علوم</v>
+        <v>لغة انجليزية</v>
       </c>
       <c r="C36" t="str">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="D36" t="str">
-        <v>(12) علوم ص٣ +(10) اسلاميات ص1 فصل 1/2 - 1/3 + ( 5 ) اسلاميات  صف 3 فصل 3/3</v>
+        <v xml:space="preserve"> (١٢) انجليزي ص١ متوسط + مكمل (١٢) حصة بالثانوي </v>
       </c>
       <c r="E36" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>عبدالعزيز الربيعان</v>
+        <v>فارس الجندي</v>
       </c>
       <c r="B37" t="str">
-        <v>اجتماعيات</v>
+        <v>علوم</v>
       </c>
       <c r="C37" t="str">
         <v>24</v>
       </c>
       <c r="D37" t="str">
-        <v xml:space="preserve">(24) اجتماعيات (9) ص١ + (9 ) ص٢ +( 6 ) ص٣ متوسط   </v>
+        <v xml:space="preserve">(12) علوم ص١ +(12) علوم ص٢ </v>
       </c>
       <c r="E37" t="str">
         <v>24</v>
@@ -12649,16 +12650,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>محمود صابر</v>
+        <v xml:space="preserve">محمد العشماوي </v>
       </c>
       <c r="B38" t="str">
-        <v>فنية</v>
+        <v>علوم</v>
       </c>
       <c r="C38" t="str">
         <v>27</v>
       </c>
       <c r="D38" t="str">
-        <v xml:space="preserve">(18) فنية ص١ ص٢ ص٣ + (9) حياتية ص١ + ص2 + ص3 فصل </v>
+        <v>(12) علوم ص٣ +(10) اسلاميات ص1 فصل 1/2 - 1/3 + ( 5 ) اسلاميات  صف 3 فصل 3/3</v>
       </c>
       <c r="E38" t="str">
         <v>27</v>
@@ -12666,50 +12667,50 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>حسين عويضة (مكمل مكرر من الثانوي)</v>
+        <v>عبدالعزيز الربيعان</v>
       </c>
       <c r="B39" t="str">
-        <v>بدنية</v>
+        <v>اجتماعيات</v>
       </c>
       <c r="C39" t="str">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D39" t="str">
-        <v>( 6) بدنية ص2 متوسط +  (6) بدنية ص٣ متوسط + مكمل (١٣) حصة بالثانوي</v>
+        <v xml:space="preserve">(24) اجتماعيات (9) ص١ + (9 ) ص٢ +( 6 ) ص٣ متوسط   </v>
       </c>
       <c r="E39" t="str">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>محمد عبد الله (مكمل مكرر من الثانوي)</v>
+        <v>محمود صابر</v>
       </c>
       <c r="B40" t="str">
-        <v>رقمية</v>
+        <v>فنية</v>
       </c>
       <c r="C40" t="str">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D40" t="str">
-        <v>(6) رقمية  ص٣ متوسط+ (2) رقمية  ص٢ متوسط فصل 3 + مكمل (١٨) حصة بالثانوي</v>
+        <v xml:space="preserve">(18) فنية ص١ ص٢ ص٣ + (9) حياتية ص١ + ص2 + ص3 فصل </v>
       </c>
       <c r="E40" t="str">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">محمود جمعه </v>
+        <v>حسين عويضة (مكمل مكرر من الثانوي)</v>
       </c>
       <c r="B41" t="str">
-        <v>رقمية</v>
+        <v>بدنية</v>
       </c>
       <c r="C41" t="str">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D41" t="str">
-        <v>(٦) رقمية  ص١متوسط +(4) رقمية  ص٢ متوسط فصل 1  + فصل 2  + ( 6) بدنية ص1 متوسط + (3) نشاط ص1 + (3) نشاط ص 3 + (3) نشاط ص2</v>
+        <v>( 6) بدنية ص2 متوسط +  (6) بدنية ص٣ متوسط + مكمل (١٣) حصة بالثانوي</v>
       </c>
       <c r="E41" t="str">
         <v>25</v>
@@ -12717,53 +12718,53 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v/>
+        <v>محمد عبد الله (مكمل مكرر من الثانوي)</v>
       </c>
       <c r="B42" t="str">
-        <v/>
+        <v>رقمية</v>
       </c>
       <c r="C42" t="str">
-        <v>315</v>
+        <v>8</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>(6) رقمية  ص٣ متوسط+ (2) رقمية  ص٢ متوسط فصل 3 + مكمل (١٨) حصة بالثانوي</v>
       </c>
       <c r="E42" t="str">
-        <v>358</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v/>
+        <v xml:space="preserve">محمود جمعه </v>
       </c>
       <c r="B43" t="str">
-        <v/>
+        <v>رقمية</v>
       </c>
       <c r="C43" t="str">
-        <v/>
+        <v>25</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>(٦) رقمية  ص١متوسط +(4) رقمية  ص٢ متوسط فصل 1  + فصل 2  + ( 6) بدنية ص1 متوسط + (3) نشاط ص1 + (3) نشاط ص 3 + (3) نشاط ص2</v>
       </c>
       <c r="E43" t="str">
-        <v/>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>اسنادات ثانوية دار القلم الفصل الدراسي الأول 1447</v>
+        <v/>
       </c>
       <c r="B44" t="str">
         <v/>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>315</v>
       </c>
       <c r="D44" t="str">
         <v/>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>358</v>
       </c>
     </row>
     <row r="45">
@@ -12785,58 +12786,58 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>المعلم</v>
+        <v/>
       </c>
       <c r="B46" t="str">
-        <v>المادة</v>
+        <v>اسنادات ثانوي (بنين)</v>
       </c>
       <c r="C46" t="str">
-        <v>عدد حصص المعلم بالمدرسة</v>
+        <v/>
       </c>
       <c r="D46" t="str">
-        <v>الإسناد</v>
+        <v/>
       </c>
       <c r="E46" t="str">
-        <v>عدد حصص المعلم بالمدرسة</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>احمد نصر</v>
+        <v/>
       </c>
       <c r="B47" t="str">
-        <v xml:space="preserve">لغة عربية </v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>24</v>
+        <v/>
       </c>
       <c r="D47" t="str">
-        <v>20 كفايات 1ث من 6:2 +4 كفايات 2ث 7</v>
+        <v/>
       </c>
       <c r="E47" t="str">
-        <v>24</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">هشام رسمي </v>
+        <v>المعلم</v>
       </c>
       <c r="B48" t="str">
-        <v xml:space="preserve">لغة عربية </v>
+        <v>المادة</v>
       </c>
       <c r="C48" t="str">
-        <v>27</v>
+        <v>عدد حصص المعلم بالمدرسة</v>
       </c>
       <c r="D48" t="str">
-        <v xml:space="preserve">24 حصة كفايات  2ث 6فصول من 6:1+ 3 حصص 2-ث نون </v>
+        <v>الإسناد</v>
       </c>
       <c r="E48" t="str">
-        <v>27</v>
+        <v>عدد حصص المعلم بالمدرسة</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">حسن الخطيب </v>
+        <v>احمد نصر</v>
       </c>
       <c r="B49" t="str">
         <v xml:space="preserve">لغة عربية </v>
@@ -12845,7 +12846,7 @@
         <v>24</v>
       </c>
       <c r="D49" t="str">
-        <v>14 مهارا ت بحث 3 ث كامل + 6 كفايات 1ث نون  +4 كفايات 1ث 1</v>
+        <v>20 كفايات 1ث من 6:2 +4 كفايات 2ث 7</v>
       </c>
       <c r="E49" t="str">
         <v>24</v>
@@ -12853,135 +12854,135 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">عبد العزيز الربيعان </v>
+        <v xml:space="preserve">هشام رسمي </v>
       </c>
       <c r="B50" t="str">
         <v xml:space="preserve">لغة عربية </v>
       </c>
       <c r="C50" t="str">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D50" t="str">
-        <v>21 تاريخ 2ث كامل+2 تاريخ 2ث نون +3 تفسير 1ث2 نون</v>
+        <v xml:space="preserve">24 حصة كفايات  2ث 6فصول من 6:1+ 3 حصص 2-ث نون </v>
       </c>
       <c r="E50" t="str">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>خالد المطيري</v>
+        <v xml:space="preserve">حسن الخطيب </v>
       </c>
       <c r="B51" t="str">
-        <v xml:space="preserve">اسلاميات </v>
+        <v xml:space="preserve">لغة عربية </v>
       </c>
       <c r="C51" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D51" t="str">
-        <v xml:space="preserve">24 تفسير وقران 1ث كامل + 3 تفسير 1ث1 نون </v>
+        <v>14 مهارا ت بحث 3 ث كامل + 6 كفايات 1ث نون  +4 كفايات 1ث 1</v>
       </c>
       <c r="E51" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">حسام السيد </v>
+        <v xml:space="preserve">عبد العزيز الربيعان </v>
       </c>
       <c r="B52" t="str">
-        <v xml:space="preserve">رياضيات </v>
+        <v xml:space="preserve">لغة عربية </v>
       </c>
       <c r="C52" t="str">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D52" t="str">
-        <v xml:space="preserve">20 صف2ث 4 فصول 4:1+4 نون صف2ث + 4 صف3ث1 </v>
+        <v>21 تاريخ 2ث كامل+2 تاريخ 2ث نون +3 تفسير 1ث2 نون</v>
       </c>
       <c r="E52" t="str">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">محمد سليم </v>
+        <v>خالد المطيري</v>
       </c>
       <c r="B53" t="str">
-        <v xml:space="preserve">رياضيات </v>
+        <v xml:space="preserve">اسلاميات </v>
       </c>
       <c r="C53" t="str">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D53" t="str">
-        <v>20صف 3ث من 6:2 +8 حصص 1 ث نون 1-2</v>
+        <v xml:space="preserve">24 تفسير وقران 1ث كامل + 3 تفسير 1ث1 نون </v>
       </c>
       <c r="E53" t="str">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">وليد الصدة </v>
+        <v xml:space="preserve">حسام السيد </v>
       </c>
       <c r="B54" t="str">
         <v xml:space="preserve">رياضيات </v>
       </c>
       <c r="C54" t="str">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D54" t="str">
-        <v xml:space="preserve">20 1ث  4 فصول من4:1+ 4 حصص 3ث7 </v>
+        <v xml:space="preserve">20 صف2ث 4 فصول 4:1+4 نون صف2ث + 4 صف3ث1 </v>
       </c>
       <c r="E54" t="str">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>وسيم عبد ربه</v>
+        <v xml:space="preserve">محمد سليم </v>
       </c>
       <c r="B55" t="str">
         <v xml:space="preserve">رياضيات </v>
       </c>
       <c r="C55" t="str">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D55" t="str">
-        <v>10 صف 1ث  6:5+ 15 صف 2ث من 7:5</v>
+        <v>20صف 3ث من 6:2 +8 حصص 1 ث نون 1-2</v>
       </c>
       <c r="E55" t="str">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">أحمد طاهر بهيدي </v>
+        <v xml:space="preserve">وليد الصدة </v>
       </c>
       <c r="B56" t="str">
-        <v xml:space="preserve">كيمياء </v>
+        <v xml:space="preserve">رياضيات </v>
       </c>
       <c r="C56" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D56" t="str">
-        <v>18 صف 1ث كامل + 6 حصص 1 ث نون 2:1 + 3 علم أرض 3ث7</v>
+        <v xml:space="preserve">20 1ث  4 فصول من4:1+ 4 حصص 3ث7 </v>
       </c>
       <c r="E56" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">أحمد محمد مصباح </v>
+        <v>وسيم عبد ربه</v>
       </c>
       <c r="B57" t="str">
-        <v xml:space="preserve">كيمياء </v>
+        <v xml:space="preserve">رياضيات </v>
       </c>
       <c r="C57" t="str">
         <v>25</v>
       </c>
       <c r="D57" t="str">
-        <v>25 حصة صف2 ث من 5:1</v>
+        <v>10 صف 1ث  6:5+ 15 صف 2ث من 7:5</v>
       </c>
       <c r="E57" t="str">
         <v>25</v>
@@ -12989,33 +12990,33 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>محمد متولي</v>
+        <v xml:space="preserve">أحمد طاهر بهيدي </v>
       </c>
       <c r="B58" t="str">
         <v xml:space="preserve">كيمياء </v>
       </c>
       <c r="C58" t="str">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D58" t="str">
-        <v>21 صف 3 ث كامل + 5 حصص 2 ث نون</v>
+        <v>18 صف 1ث كامل + 6 حصص 1 ث نون 2:1 + 3 علم أرض 3ث7</v>
       </c>
       <c r="E58" t="str">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>حسن جوده</v>
+        <v xml:space="preserve">أحمد محمد مصباح </v>
       </c>
       <c r="B59" t="str">
-        <v>كيمياء - فيزياء</v>
+        <v xml:space="preserve">كيمياء </v>
       </c>
       <c r="C59" t="str">
         <v>25</v>
       </c>
       <c r="D59" t="str">
-        <v>10كيمياء  صف 2ث 7:6+15فيزياء  صف 3ث 3:1</v>
+        <v>25 حصة صف2 ث من 5:1</v>
       </c>
       <c r="E59" t="str">
         <v>25</v>
@@ -13023,75 +13024,75 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>فريج السعيد</v>
+        <v>محمد متولي</v>
       </c>
       <c r="B60" t="str">
-        <v xml:space="preserve">فيزياء </v>
+        <v xml:space="preserve">كيمياء </v>
       </c>
       <c r="C60" t="str">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D60" t="str">
-        <v xml:space="preserve"> 20صف 3ث 7:4 + 4 حصص 2 ث7</v>
+        <v>21 صف 3 ث كامل + 5 حصص 2 ث نون</v>
       </c>
       <c r="E60" t="str">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">سلمان محمد </v>
+        <v>حسن جوده</v>
       </c>
       <c r="B61" t="str">
-        <v xml:space="preserve">فيزياء </v>
+        <v>كيمياء - فيزياء</v>
       </c>
       <c r="C61" t="str">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D61" t="str">
-        <v xml:space="preserve">24 حصة صف2 ث 6 فصول 6:1 + 4 حصص 2ث نون </v>
+        <v>10كيمياء  صف 2ث 7:6+15فيزياء  صف 3ث 3:1</v>
       </c>
       <c r="E61" t="str">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">محمد عبد المنعم </v>
+        <v>فريج السعيد</v>
       </c>
       <c r="B62" t="str">
-        <v xml:space="preserve">أحياء </v>
+        <v xml:space="preserve">فيزياء </v>
       </c>
       <c r="C62" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D62" t="str">
-        <v>18 صف 1ث كامل + 3 علم ارض ص ثالث6 +6 حصص 1 ث نون 1و2</v>
+        <v xml:space="preserve"> 20صف 3ث 7:4 + 4 حصص 2 ث7</v>
       </c>
       <c r="E62" t="str">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>حسن ابوغنيمة</v>
+        <v xml:space="preserve">سلمان محمد </v>
       </c>
       <c r="B63" t="str">
-        <v xml:space="preserve">أحياء </v>
+        <v xml:space="preserve">فيزياء </v>
       </c>
       <c r="C63" t="str">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D63" t="str">
-        <v>20 حصة 2ث 4:1+4أحياء  2ث نون+ مسند له كلاسيرا</v>
+        <v xml:space="preserve">24 حصة صف2 ث 6 فصول 6:1 + 4 حصص 2ث نون </v>
       </c>
       <c r="E63" t="str">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>محمد علي</v>
+        <v xml:space="preserve">محمد عبد المنعم </v>
       </c>
       <c r="B64" t="str">
         <v xml:space="preserve">أحياء </v>
@@ -13100,7 +13101,7 @@
         <v>27</v>
       </c>
       <c r="D64" t="str">
-        <v>15 علم أرض 3ث من 5:3 + 12 أحياءص2ث 7:5</v>
+        <v>18 صف 1ث كامل + 3 علم ارض ص ثالث6 +6 حصص 1 ث نون 1و2</v>
       </c>
       <c r="E64" t="str">
         <v>27</v>
@@ -13108,84 +13109,84 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v xml:space="preserve">مصطفى محمد </v>
+        <v>حسن ابوغنيمة</v>
       </c>
       <c r="B65" t="str">
-        <v xml:space="preserve">لغة انجليزية </v>
+        <v xml:space="preserve">أحياء </v>
       </c>
       <c r="C65" t="str">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D65" t="str">
-        <v>24حصة اث كامل + 2 حصة 1ث نون 1</v>
+        <v>20 حصة 2ث 4:1+4أحياء  2ث نون+ مسند له كلاسيرا</v>
       </c>
       <c r="E65" t="str">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">عبد الرحمن شطا </v>
+        <v>محمد علي</v>
       </c>
       <c r="B66" t="str">
-        <v xml:space="preserve">لغة انجليزية </v>
+        <v xml:space="preserve">أحياء </v>
       </c>
       <c r="C66" t="str">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D66" t="str">
-        <v>20حصة 2 ث من5:1+ 4 حصص 3ث1+ 1 حصة نون 2ث</v>
+        <v>15 علم أرض 3ث من 5:3 + 12 أحياءص2ث 7:5</v>
       </c>
       <c r="E66" t="str">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">مصطفى فتحي (مكرر مكمل من المتوسط) </v>
+        <v xml:space="preserve">مصطفى محمد </v>
       </c>
       <c r="B67" t="str">
         <v xml:space="preserve">لغة انجليزية </v>
       </c>
       <c r="C67" t="str">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D67" t="str">
-        <v>8 حصص 2 ث 6 و7 + 4 تفكير ناقد صف 1ث نون 1و2 + مكمل (١٢) حصة بالمتوسط</v>
+        <v>24حصة اث كامل + 2 حصة 1ث نون 1</v>
       </c>
       <c r="E67" t="str">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>إبراهيم شبكة</v>
+        <v xml:space="preserve">عبد الرحمن شطا </v>
       </c>
       <c r="B68" t="str">
         <v xml:space="preserve">لغة انجليزية </v>
       </c>
       <c r="C68" t="str">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D68" t="str">
-        <v>24 حصة صف 3ث 7:2</v>
+        <v>20حصة 2 ث من5:1+ 4 حصص 3ث1+ 1 حصة نون 2ث</v>
       </c>
       <c r="E68" t="str">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>احمد توفيق</v>
+        <v xml:space="preserve">مصطفى فتحي (مكرر مكمل من المتوسط) </v>
       </c>
       <c r="B69" t="str">
-        <v>تقنية -حاسب</v>
+        <v xml:space="preserve">لغة انجليزية </v>
       </c>
       <c r="C69" t="str">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D69" t="str">
-        <v>20 حصة مجال صف 3 ث 5:1+ 4 حصص 1ث نون تقنية 1و2</v>
+        <v>8 حصص 2 ث 6 و7 + 4 تفكير ناقد صف 1ث نون 1و2 + مكمل (١٢) حصة بالمتوسط</v>
       </c>
       <c r="E69" t="str">
         <v>24</v>
@@ -13193,16 +13194,16 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v xml:space="preserve">محمد مدحت </v>
+        <v>إبراهيم شبكة</v>
       </c>
       <c r="B70" t="str">
-        <v>تقنية -حاسب</v>
+        <v xml:space="preserve">لغة انجليزية </v>
       </c>
       <c r="C70" t="str">
         <v>24</v>
       </c>
       <c r="D70" t="str">
-        <v xml:space="preserve">18 حصة 1ث كامل  + 6تفكير ناقد 1ث </v>
+        <v>24 حصة صف 3ث 7:2</v>
       </c>
       <c r="E70" t="str">
         <v>24</v>
@@ -13210,83 +13211,117 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v xml:space="preserve">محمد صلاح </v>
+        <v>احمد توفيق</v>
       </c>
       <c r="B71" t="str">
-        <v xml:space="preserve">بدنية </v>
+        <v>تقنية -حاسب</v>
       </c>
       <c r="C71" t="str">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D71" t="str">
-        <v>12حصة 1ث كامل+12بدنية 3ث من  4:1 + 4 صف اول نون 1و2</v>
+        <v>20 حصة مجال صف 3 ث 5:1+ 4 حصص 1ث نون تقنية 1و2</v>
       </c>
       <c r="E71" t="str">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v xml:space="preserve">حسين عويضة </v>
+        <v xml:space="preserve">محمد مدحت </v>
       </c>
       <c r="B72" t="str">
-        <v xml:space="preserve">بدنية </v>
+        <v>تقنية -حاسب</v>
       </c>
       <c r="C72" t="str">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D72" t="str">
-        <v>9بدنية 3ث 7:5 + 8 مجال اختياري 3ث6 (م بالمتوسط بعد الفسحة) + مكمل (١٢) حصة بالمتوسط</v>
+        <v xml:space="preserve">18 حصة 1ث كامل  + 6تفكير ناقد 1ث </v>
       </c>
       <c r="E72" t="str">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v xml:space="preserve">عيد العتيبي + (م .اداري)   </v>
+        <v xml:space="preserve">محمد صلاح </v>
       </c>
       <c r="B73" t="str">
-        <v xml:space="preserve">علم نفس </v>
+        <v xml:space="preserve">بدنية </v>
       </c>
       <c r="C73" t="str">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D73" t="str">
-        <v xml:space="preserve"> 6 تفكير ناقد 1ث+ 7 نشاط 2ث + مكمل مراقب دور</v>
+        <v>12حصة 1ث كامل+12بدنية 3ث من  4:1 + 4 صف اول نون 1و2</v>
       </c>
       <c r="E73" t="str">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
+        <v xml:space="preserve">حسين عويضة </v>
+      </c>
+      <c r="B74" t="str">
+        <v xml:space="preserve">بدنية </v>
+      </c>
+      <c r="C74" t="str">
+        <v>13</v>
+      </c>
+      <c r="D74" t="str">
+        <v>9بدنية 3ث 7:5 + 8 مجال اختياري 3ث6 (م بالمتوسط بعد الفسحة) + مكمل (١٢) حصة بالمتوسط</v>
+      </c>
+      <c r="E74" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v xml:space="preserve">عيد العتيبي + (م .اداري)   </v>
+      </c>
+      <c r="B75" t="str">
+        <v xml:space="preserve">علم نفس </v>
+      </c>
+      <c r="C75" t="str">
+        <v>13</v>
+      </c>
+      <c r="D75" t="str">
+        <v xml:space="preserve"> 6 تفكير ناقد 1ث+ 7 نشاط 2ث + مكمل مراقب دور</v>
+      </c>
+      <c r="E75" t="str">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
         <v>محمد عبد الله</v>
       </c>
-      <c r="B74" t="str">
+      <c r="B76" t="str">
         <v>تقنية -حاسب</v>
       </c>
-      <c r="C74" t="str">
+      <c r="C76" t="str">
         <v>18</v>
       </c>
-      <c r="D74" t="str">
+      <c r="D76" t="str">
         <v>14 تقنية 3ث كامل + 4 مجال صف 3 ث 7+ مكمل (٨) حصص بالمتوسط</v>
       </c>
-      <c r="E74" t="str">
+      <c r="E76" t="str">
         <v>26</v>
       </c>
     </row>
-    <row r="75" xml:space="preserve">
-      <c r="A75" t="str">
+    <row r="77" xml:space="preserve">
+      <c r="A77" t="str">
         <v>إجمالي الحصص</v>
       </c>
-      <c r="B75" t="str">
-        <v/>
-      </c>
-      <c r="C75" t="str">
-        <v/>
-      </c>
-      <c r="D75" t="str" xml:space="preserve">
+      <c r="B77" t="str">
+        <v/>
+      </c>
+      <c r="C77" t="str">
+        <v/>
+      </c>
+      <c r="D77" t="str" xml:space="preserve">
         <v xml:space="preserve">تخفيض حصة من اللغة الإنجليزية أول ثانوي_x000d_
 تخفيض حصة من اللغة الإنجليزيةوثان _x000d_
 تخفيض حصة تفكير ناقد أول ثانوي _x000d_
@@ -13295,18 +13330,965 @@
 تخفيض حصة مجال صف ثالث ثانوي _x000d_
 عليه خروج جميع طلاب المدرسة بعد الحصة السادسة يوميا 11:50( بواقع تخفيض حصتين من كل فصل ) </v>
       </c>
-      <c r="E75" t="str">
+      <c r="E77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v/>
+      </c>
+      <c r="B78" t="str">
+        <v/>
+      </c>
+      <c r="C78" t="str">
+        <v/>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v/>
+      </c>
+      <c r="B79" t="str">
+        <v>========================================</v>
+      </c>
+      <c r="C79" t="str">
+        <v/>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v>اسنادات قطاع البنات</v>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v/>
+      </c>
+      <c r="B81" t="str">
+        <v/>
+      </c>
+      <c r="C81" t="str">
+        <v/>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v/>
+      </c>
+      <c r="B82" t="str">
+        <v>اسنادات ابتدائي (بنات)</v>
+      </c>
+      <c r="C82" t="str">
+        <v/>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B83" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C83" t="str">
+        <v xml:space="preserve">عدد حصص المعلم بالمرحلة </v>
+      </c>
+      <c r="D83" t="str">
+        <v>ملاحظات</v>
+      </c>
+      <c r="E83" t="str">
+        <v>إجمالي نصاب المعلم بعد الاكمال</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v/>
+      </c>
+      <c r="B84" t="str">
+        <v/>
+      </c>
+      <c r="C84" t="str">
+        <v/>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v xml:space="preserve">نورا مجدي </v>
+      </c>
+      <c r="B85" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C85">
+        <v>24</v>
+      </c>
+      <c r="D85" t="str">
+        <v>(3) انجليزي وزاري ص1 ( 2) انجليزي اثرائي ص1 (1) ماث ص1 ( 1) ساينس ص1 ( 3) انجليزي وزاري ص2 (2) انجليزي اثرائي ص2 (6) انجليزي وزاري ص3 (4)انجليزي اثرائي ص3 (2) نشاط ص5</v>
+      </c>
+      <c r="E85">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v xml:space="preserve">سارة المخلفي </v>
+      </c>
+      <c r="B86" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C86">
+        <v>24</v>
+      </c>
+      <c r="D86" t="str">
+        <v>(10)اسلاميةص3(5)اسلاميةص4(5)إسلامية ص5(2)اجتماعيات ص5(2)نشاط ص4 + منسقة تطوع ابتدائي ومتوسط</v>
+      </c>
+      <c r="E86">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>نوير الشمري ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B87" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C87">
+        <v>8</v>
+      </c>
+      <c r="D87" t="str">
+        <v>(2) رقمية ص2 (2)رقمية ص4(2)رقمية ص5(2) رقمية ص6 + مسند (٦) حصص بالمتوسط + (10) حصة بالثانوي</v>
+      </c>
+      <c r="E87">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>نهال الشبرمي ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B88" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C88">
+        <v>7</v>
+      </c>
+      <c r="D88" t="str">
+        <v>(2) بدنية ص6 (5) إسلامية ص6 + مسند (13) حصة بالمتوسط + (4) رقمية kg + منسقة الصيانة والمشتريات</v>
+      </c>
+      <c r="E88">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v xml:space="preserve">نوضا المطيري </v>
+      </c>
+      <c r="B89" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C89">
+        <v>24</v>
+      </c>
+      <c r="D89" t="str">
+        <v>(4)رياضيات ص1(3) علوم ص1 (3) علوم ص2 (6) رياضيات ص4 (2)اجتماعايت ص4 (1) اسرية ص4(1) نشاط ص3 فصل(4) رقمية ص3</v>
+      </c>
+      <c r="E89">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>الجوهرة المخلفي  ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B90" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C90">
+        <v>7</v>
+      </c>
+      <c r="D90" t="str">
+        <v>(5) لغتي ص6 (2) اجتماعيات ص6 + (17) حصة بالمتوسط + منسقة اختبارات مركزية</v>
+      </c>
+      <c r="E90">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>حنان العنزي (مكرر مكمل من متوسط )</v>
+      </c>
+      <c r="B91" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91" t="str">
+        <v>(3) بدنية ص1 + مسند لها ( 11 ) متوسط + (11) ثانوي + منسقة اختبارات steep</v>
+      </c>
+      <c r="E91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>أشواق العنزي</v>
+      </c>
+      <c r="B92" t="str">
+        <v xml:space="preserve"> لغة عربية</v>
+      </c>
+      <c r="C92">
+        <v>25</v>
+      </c>
+      <c r="D92" t="str">
+        <v>(8)لغتي ص1 (7)لغتي ص2 (5) إسلامية ص1(5) إسلامية ص2</v>
+      </c>
+      <c r="E92">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>ناهد بعزقي</v>
+      </c>
+      <c r="B93" t="str">
+        <v xml:space="preserve"> لغة عربية</v>
+      </c>
+      <c r="C93">
+        <v>24</v>
+      </c>
+      <c r="D93" t="str">
+        <v>(12) لغتي ص3 (5)لغتي ص4 (5) لغتي ص5 (1)اسرية ص5 (1) نشاط ص 3فصل</v>
+      </c>
+      <c r="E93">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>نوف الزلفي</v>
+      </c>
+      <c r="B94" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C94">
+        <v>24</v>
+      </c>
+      <c r="D94" t="str">
+        <v>(6)رياضيات ص2 (12) رياضيات ص3 (6) بدنية ص3 + معلمة موهبة</v>
+      </c>
+      <c r="E94">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>نور العيدة ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B95" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C95">
+        <v>6</v>
+      </c>
+      <c r="D95" t="str">
+        <v xml:space="preserve"> ( 6 )  رياضيات ص6 + مسند ( 18) ثانوي + منسقة قدرات وتحصيلي</v>
+      </c>
+      <c r="E95">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>هدى المطيري ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B96" t="str">
+        <v>كيمياء</v>
+      </c>
+      <c r="C96">
+        <v>2</v>
+      </c>
+      <c r="D96" t="str">
+        <v>(2) بدنية ص5 + مسند ( 23) ثانوي</v>
+      </c>
+      <c r="E96">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>سلطانة العتيبي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B97" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C97">
+        <v>1</v>
+      </c>
+      <c r="D97" t="str">
+        <v>(1) اسرية ص6 + ( 18 ) ثانوي + ( 5) متوسط</v>
+      </c>
+      <c r="E97">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>نوف العتيبي ( مكرر مكمل من الثانوي )</v>
+      </c>
+      <c r="B98" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C98">
+        <v>2</v>
+      </c>
+      <c r="D98" t="str">
+        <v>(2) رقمية ص1 + (22) مسند ثانوي</v>
+      </c>
+      <c r="E98">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>بدور  البقمي  ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B99" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C99">
+        <v>6</v>
+      </c>
+      <c r="D99" t="str">
+        <v>(6)رياضيات ص5 + مسند ( 18)  متوسط</v>
+      </c>
+      <c r="E99">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>منى الخلف</v>
+      </c>
+      <c r="B100" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C100">
+        <v>20</v>
+      </c>
+      <c r="D100" t="str">
+        <v xml:space="preserve"> (8) علوم ص3 (4) علوم ص4 (4) علوم ص5  (4) علوم ص6 + مسند (4) بالمتوسط</v>
+      </c>
+      <c r="E100">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v xml:space="preserve"> عهود الرويلي </v>
+      </c>
+      <c r="B101" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C101">
+        <v>20</v>
+      </c>
+      <c r="D101" t="str">
+        <v>(3) انجليزي وزاري ص4 ( 2) انجليزي اثرائي ص4  ( 3) انجليزي وزاري ص5 (2) انجليزي اثرائي ص5 (3) انجليزي وزاري ص6 (2)انجليزي اثرائي ص6 (3) بدنية ص2 (2) نشاط ص6 + (4) kg</v>
+      </c>
+      <c r="E101">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v xml:space="preserve">هدى البكري </v>
+      </c>
+      <c r="B102" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C102">
+        <v>18</v>
+      </c>
+      <c r="D102" t="str">
+        <v>(2)فنية ص1(2) فنية ص2(4) فنية ص3(1) فنية ص4(1)فنية ص5(1) قنية ص6  (2) بدنية ص4 (1)نشاط ص2 (1) اسرية ص1(1) اسرية ص2(2)اسرية ص3+ مسند (6) حصص بالمتوسط + موجهة صحية ابتدائي</v>
+      </c>
+      <c r="E102">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B103">
+        <v>245</v>
+      </c>
+      <c r="C103">
+        <v>245</v>
+      </c>
+      <c r="D103" t="str">
+        <v>تم زيادة ( 14) حصة لتفعيل المواد الاثرائية ورفع مستوى التحصيل فأصبح إجمالي الحصص في الأسبوع 35</v>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v/>
+      </c>
+      <c r="B104" t="str">
+        <v>اسنادات متوسط (بنات)</v>
+      </c>
+      <c r="C104" t="str">
+        <v/>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B105" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C105" t="str">
+        <v xml:space="preserve">عدد حصص المعلم بالمرحلة </v>
+      </c>
+      <c r="D105" t="str">
+        <v>ملاحظات</v>
+      </c>
+      <c r="E105" t="str">
+        <v>إجمالي نصاب المعلم بعد الاكمال</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v/>
+      </c>
+      <c r="B106" t="str">
+        <v/>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>هدى البكري ( مكرر مكمل من ابتدائي)</v>
+      </c>
+      <c r="B107" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C107">
+        <v>6</v>
+      </c>
+      <c r="D107" t="str">
+        <v>(2) فنية ص1 (2) فنية ص2 (2) فنية ص + مسند (18) حصة بالابتدائي + موجهة صحية ابتدائي</v>
+      </c>
+      <c r="E107">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v xml:space="preserve">حنان الغربي </v>
+      </c>
+      <c r="B108" t="str">
+        <v>اجتماعيات</v>
+      </c>
+      <c r="C108">
+        <v>11</v>
+      </c>
+      <c r="D108" t="str">
+        <v>(3) اجتماعيات ص1 (3) اجتماعيات ص2(2) اجتماعيات ص3 (2) بدنية 3م (1) اسرية 3م + مسند (13) حصص بالثانوي + مسؤولة المقصف</v>
+      </c>
+      <c r="E108">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>نوير الشمري    ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B109" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C109">
+        <v>6</v>
+      </c>
+      <c r="D109" t="str">
+        <v>(2) رقمية ص1 (2) رقمية ص3 (2) رقمية ص3 + مسند (١0) حصص بالثانوي + (8) حصص بالابتدائي</v>
+      </c>
+      <c r="E109">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>منى الخلف ( مكرر مكمل من الابتدائي )</v>
+      </c>
+      <c r="B110" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C110">
+        <v>4</v>
+      </c>
+      <c r="D110" t="str">
+        <v>(4) علوم ص1 + مسند (20 ) ابتدائي</v>
+      </c>
+      <c r="E110">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>بدور  البقمي</v>
+      </c>
+      <c r="B111" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C111">
+        <v>18</v>
+      </c>
+      <c r="D111" t="str">
+        <v>(6) رياضيات ص1 (6) رياضيات ص2 (6) رياضيات ص3 + مسند لها (6) ابتدائي</v>
+      </c>
+      <c r="E111">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>ريم الحربي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B112" t="str">
+        <v>دين</v>
+      </c>
+      <c r="C112">
+        <v>5</v>
+      </c>
+      <c r="D112" t="str">
+        <v>( 5 ) إسلامية ص3 + مسند ثانوي 19 ثانوي</v>
+      </c>
+      <c r="E112">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>اماني فهمي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B113" t="str">
+        <v>احياء</v>
+      </c>
+      <c r="C113">
+        <v>4</v>
+      </c>
+      <c r="D113" t="str">
+        <v>(4) علوم ص2 + مسند لها (20) ثانوي</v>
+      </c>
+      <c r="E113">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>سلطانة العتيبي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B114" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C114">
+        <v>5</v>
+      </c>
+      <c r="D114" t="str">
+        <v>(4) علوم ص3 (1) نشاط ص3 + مسند لها (18 ) ثانوي + ( 1) ابتدائي + منسقة نافس</v>
+      </c>
+      <c r="E114">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>امل العنزي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B115" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C115">
+        <v>5</v>
+      </c>
+      <c r="D115" t="str">
+        <v>(4) انجليزي ص3 (1) أسرية ص3 + مسند (19) حصة بالثانوي + منسقة اختبارات steep</v>
+      </c>
+      <c r="E115">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>حنان العنزي</v>
+      </c>
+      <c r="B116" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C116">
+        <v>11</v>
+      </c>
+      <c r="D116" t="str">
+        <v>(4) انجليزي ص1(4) انجليزي ص2(1)اسرية ص2 (2) بدنية ص2+ مسند لها (11) حصة ثانوي+(3) ابتدائي</v>
+      </c>
+      <c r="E116">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>الجوهرة المخلفي</v>
+      </c>
+      <c r="B117" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C117">
+        <v>17</v>
+      </c>
+      <c r="D117" t="str">
+        <v>(5) لغتي ص1 (5) لغتي ص2(4) لغتي ص3 (2) بدنية ص1 (1) نشاط ص1 + مسند (7) حصص بالابتدائي + منسقة اختبارات مركزية</v>
+      </c>
+      <c r="E117">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>نهال الشبرمي</v>
+      </c>
+      <c r="B118" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C118">
+        <v>13</v>
+      </c>
+      <c r="D118" t="str">
+        <v>(5) إسلامية ص1 (5) إسلامية ص2  (٢)  تفكير ناقد ص3  (1) نشاط ص2 + مسند (7) حصص بالابتدائي + (4) kg + منسقة الصيانة والمشتريات</v>
+      </c>
+      <c r="E118">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B119">
+        <v>105</v>
+      </c>
+      <c r="C119">
+        <v>105</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v/>
+      </c>
+      <c r="B120" t="str">
+        <v>اسنادات ثانوي (بنات)</v>
+      </c>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B121" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C121" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+      <c r="D121" t="str">
+        <v>الإسناد</v>
+      </c>
+      <c r="E121" t="str">
+        <v>إجمالي نصاب المعلم</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>حنان الغربي ( مكرر مكمل  متوسط )</v>
+      </c>
+      <c r="B122" t="str">
+        <v>اجتماعيات</v>
+      </c>
+      <c r="C122">
+        <v>13</v>
+      </c>
+      <c r="D122" t="str">
+        <v>(6) تاريخ ص2 (6) بدنية ص3 (1) نشاط ص3 فصل + مسند (11) حصص بالمتوسط + مسؤولة المقصف</v>
+      </c>
+      <c r="E122">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v xml:space="preserve">نوف العتيبي </v>
+      </c>
+      <c r="B123" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C123">
+        <v>22</v>
+      </c>
+      <c r="D123" t="str">
+        <v>(8) كفايات ص1(8) كفايات ص2 (4) بحث ومعلومات ص3 (2) نشاط ص2  + مسند (2) ابتدائي + أمينة مصادر</v>
+      </c>
+      <c r="E123">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>ريم الحربي</v>
+      </c>
+      <c r="B124" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C124">
+        <v>19</v>
+      </c>
+      <c r="D124" t="str">
+        <v>(6) تفكير ناقد ص1 (8) قرآن وتفسيره صف1 (5) مجال اختياري مهارات إدارية + مسند (5) متوسط</v>
+      </c>
+      <c r="E124">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>سلطانة البقمي</v>
+      </c>
+      <c r="B125" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C125">
+        <v>25</v>
+      </c>
+      <c r="D125" t="str">
+        <v xml:space="preserve">(8) رياضيات ص3 (10) رياضيات ص1 ( 4) بدنية ص1 (3) نشاط ص3 </v>
+      </c>
+      <c r="E125">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>نور العيدة</v>
+      </c>
+      <c r="B126" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C126">
+        <v>18</v>
+      </c>
+      <c r="D126" t="str">
+        <v>(10) رياضيات ص2 (3) نشاط ص2 (5) مجال اختياري تنمية مستدامة ص3 + مسند (6) ابتدائي+ منسقة قدرات وتحصيلي</v>
+      </c>
+      <c r="E126">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>سلطانة العتيبي</v>
+      </c>
+      <c r="B127" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C127">
+        <v>18</v>
+      </c>
+      <c r="D127" t="str">
+        <v>(8) فيزياء ص2 (10) فيزياء ص3 + مسند (5) متوسط + (1) ابتدائي  + منسقة نافس</v>
+      </c>
+      <c r="E127">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>هدى المطيري</v>
+      </c>
+      <c r="B128" t="str">
+        <v>كيمياء</v>
+      </c>
+      <c r="C128">
+        <v>23</v>
+      </c>
+      <c r="D128" t="str">
+        <v>(6) كيمياء ص1 (10) كيمياء ص2 (6) كيمياء ص3 (1) نشاط ص1 فصل + (2) مسند ابتدائي</v>
+      </c>
+      <c r="E128">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>أماني فهمي</v>
+      </c>
+      <c r="B129" t="str">
+        <v>أحياء</v>
+      </c>
+      <c r="C129">
+        <v>20</v>
+      </c>
+      <c r="D129" t="str">
+        <v>(6) أحياء ص1 (8) أحياء ص2 (9) علم الأرض ص3 + مسند (4) متوسط</v>
+      </c>
+      <c r="E129">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>حنان العنزي (مكرر مكمل من متوسط )</v>
+      </c>
+      <c r="B130" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C130">
+        <v>11</v>
+      </c>
+      <c r="D130" t="str">
+        <v>(10) انجليزي ص1 (1) نشاط ص1 فصل + مسند (11) متوسط +( 3) ابتدائي</v>
+      </c>
+      <c r="E130">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v xml:space="preserve">أمل العنزي </v>
+      </c>
+      <c r="B131" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C131">
+        <v>19</v>
+      </c>
+      <c r="D131" t="str">
+        <v>(8) انجليزي ص3 (10) انجليزي ص2 (1) نشاط ص2 فصل + مسند (5) متوسط + منسقة اختبارات steep</v>
+      </c>
+      <c r="E131">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v xml:space="preserve">نوير الشمري </v>
+      </c>
+      <c r="B132" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C132">
+        <v>10</v>
+      </c>
+      <c r="D132" t="str">
+        <v>(٦) تقنية رقمية ص1 (4) رقمية ص3  + مسند (٦) حصص بالمتوسط + (8) حصص بالابتدائي</v>
+      </c>
+      <c r="E132">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B133">
+        <v>198</v>
+      </c>
+      <c r="C133">
+        <v>198</v>
+      </c>
+      <c r="D133" t="str">
+        <v>تم زيادة ( 6) حصص لتفعيل البرامج الاثرائية ورفع مستوى التحصيل فأصبحت إجمالي الحصص 198</v>
+      </c>
+      <c r="E133" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A44:E44"/>
-  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E133"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -18797,6 +19779,2291 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E133"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v/>
+      </c>
+      <c r="B1" t="str">
+        <v>اسنادات قطاع البنين</v>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>اسنادات ابتدائي (بنين)</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B6" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C6" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+      <c r="D6" t="str">
+        <v>الإسناد</v>
+      </c>
+      <c r="E6" t="str">
+        <v>إجمالي نصاب المعلم</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>العفيفي عبد الجواد</v>
+      </c>
+      <c r="B7" t="str">
+        <v>معلم صف أول</v>
+      </c>
+      <c r="C7" t="str">
+        <v>24</v>
+      </c>
+      <c r="D7" t="str">
+        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>محمود عبدالحسيب</v>
+      </c>
+      <c r="B8" t="str">
+        <v>معلم صف أول</v>
+      </c>
+      <c r="C8" t="str">
+        <v>24</v>
+      </c>
+      <c r="D8" t="str">
+        <v>(٨) لغتي ص١+ (٤) اسلاميات ص١+ (٥) رياضيات ص١+ (٢) بدنية ص١+ (١) مهارات حياتية ص١ + (1) فنية ص١ + (3) علوم ص1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>عبد العزيز يونس</v>
+      </c>
+      <c r="B9" t="str">
+        <v>معلم صف ثاني</v>
+      </c>
+      <c r="C9" t="str">
+        <v>24</v>
+      </c>
+      <c r="D9" t="str">
+        <v xml:space="preserve">(١٤) لغتي ص٢ فصلين + (١٠) اسلاميات ص٢ فصلين </v>
+      </c>
+      <c r="E9" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>حسن عزالدين مبروك</v>
+      </c>
+      <c r="B10" t="str">
+        <v>معلم صف ثالث</v>
+      </c>
+      <c r="C10" t="str">
+        <v>24</v>
+      </c>
+      <c r="D10" t="str">
+        <v>(١٤) لغتي ص٣ فصلين(2/4 ، 3/4) + (١٠) اسلاميات ص٣ فصلين +(٢) مهارات حياتية ص٣ فصلين</v>
+      </c>
+      <c r="E10" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>سلمان حمد الفراج</v>
+      </c>
+      <c r="B11" t="str">
+        <v>اسلاميات</v>
+      </c>
+      <c r="C11" t="str">
+        <v>24</v>
+      </c>
+      <c r="D11" t="str">
+        <v>(١٢) اسلاميات ص٤ فصلين (2/4 ،3/4)+ (٨) اسلاميات ص٥+ (٤) اسلاميات ص٦ فصلين</v>
+      </c>
+      <c r="E11" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>محمد الغباشي</v>
+      </c>
+      <c r="B12" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C12" t="str">
+        <v>25</v>
+      </c>
+      <c r="D12" t="str">
+        <v>(٥) لغتي ص 4 فصل(2/4) + (١٠) لغتي ص٥ فصلين +(١٠) لغتي ص٦ فصلين</v>
+      </c>
+      <c r="E12" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>طارق عبدالظاهر</v>
+      </c>
+      <c r="B13" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C13" t="str">
+        <v>24</v>
+      </c>
+      <c r="D13" t="str">
+        <v>(18) رياضيات ص٤ +(6) رياضيات ص٥ فصل</v>
+      </c>
+      <c r="E13" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v xml:space="preserve">احمد سالم </v>
+      </c>
+      <c r="B14" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C14" t="str">
+        <v>24</v>
+      </c>
+      <c r="D14" t="str">
+        <v>(١٢) رياضيات ص٦ فصلين  + مسند (6) رياضيات ص5 فصل + (5) نشاط ص4 وص5 + (1) نشاط ص6 فصل</v>
+      </c>
+      <c r="E14" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">عمرو محمد </v>
+      </c>
+      <c r="B15" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C15" t="str">
+        <v>24</v>
+      </c>
+      <c r="D15" t="str">
+        <v xml:space="preserve">(12) رياضيات ص٢ ب فصلين+(12) رياضيات ص٣ فصلين </v>
+      </c>
+      <c r="E15" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ربيع عوض</v>
+      </c>
+      <c r="B16" t="str">
+        <v>لغة انجليزية</v>
+      </c>
+      <c r="C16" t="str">
+        <v>24</v>
+      </c>
+      <c r="D16" t="str">
+        <v>(٦) E ص٥ + (٦) E ص٦ + (٩) E ص٤ + (2) انجليزي إثرائي ص6 + (1) نشاط ص6 فصل</v>
+      </c>
+      <c r="E16" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>محمد السيد</v>
+      </c>
+      <c r="B17" t="str">
+        <v>لغة انجليزية</v>
+      </c>
+      <c r="C17" t="str">
+        <v>24</v>
+      </c>
+      <c r="D17" t="str">
+        <v xml:space="preserve"> (٦) E ص٣ + + (٤) E اثرائي ص3  + (٦) E اثرائي ص٤ + (2) E اثرائي ص٦+ (٤) E اثراىي ص٥ +(2) انجليزي اثرائي ص2 فصل</v>
+      </c>
+      <c r="E17" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>احمد حسنين</v>
+      </c>
+      <c r="B18" t="str">
+        <v>لغة انجليزية</v>
+      </c>
+      <c r="C18" t="str">
+        <v>24</v>
+      </c>
+      <c r="D18" t="str">
+        <v>(6) E ص١+ (٤) E اثرائي ص١+ (٦) E ص٢ + (2) E اثرائي ص٢ فصل+ (4) ماث ص١ + (٢) ساينس ص١</v>
+      </c>
+      <c r="E18" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v xml:space="preserve"> ايمن محمد </v>
+      </c>
+      <c r="B19" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C19" t="str">
+        <v>24</v>
+      </c>
+      <c r="D19" t="str">
+        <v>(٦) علوم ص2 فصلين+ (8) علوم ص٣ فصلين+ (٨) علوم ص4 فصلين(1/4،2/4)+ (٢) بدنية ص5 فصل (2/5)</v>
+      </c>
+      <c r="E19" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>مصطفى عبدالتواب</v>
+      </c>
+      <c r="B20" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C20" t="str">
+        <v>24</v>
+      </c>
+      <c r="D20" t="str">
+        <v>(٨) علوم ص٥  + (٨) علوم ص٦ + (٤) علوم ص٤ + (٤) اجتماعيات ص٦</v>
+      </c>
+      <c r="E20" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>محمد إبراهيم</v>
+      </c>
+      <c r="B21" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C21" t="str">
+        <v>24</v>
+      </c>
+      <c r="D21" t="str">
+        <v>(١٠) لغتي ص٤ فصلين(1/4،3/4) + (٤) اسلاميات ص4 فصل(1/4) + (١٠) اجتماعيات ص٤ فصلين ص٥ فصلين</v>
+      </c>
+      <c r="E21" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>رامي يسن معروف</v>
+      </c>
+      <c r="B22" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C22" t="str">
+        <v>24</v>
+      </c>
+      <c r="D22" t="str">
+        <v>(٤) فنية ص٢+ (٤) فنية ص٣ + (٣) فنية ص٤ + (٢) فنية ص٥ + (٢) فنية ص٦ + (٩) مهارات حياتية ص٢، ص٤، ص٥، ص٦</v>
+      </c>
+      <c r="E22" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>محمود وحش</v>
+      </c>
+      <c r="B23" t="str">
+        <v>بدنية</v>
+      </c>
+      <c r="C23" t="str">
+        <v>24</v>
+      </c>
+      <c r="D23" t="str">
+        <v>(6) بدنية ص٣ + (٦) بدنية ص٤ + (6) بدنية ص٢  + (2) بدنية ص٥ +  (4) بدنية ص6</v>
+      </c>
+      <c r="E23" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>آمير جلال</v>
+      </c>
+      <c r="B24" t="str">
+        <v>رقمية</v>
+      </c>
+      <c r="C24" t="str">
+        <v>24</v>
+      </c>
+      <c r="D24" t="str">
+        <v xml:space="preserve">(2) رقمية ص١+ (٤) رقمية ص٢+ (٤) رقمية ص٣ + (٦) رقمية ص٤ + (٤) رقمية ص٥ + (٤) رقمية ص٦ </v>
+      </c>
+      <c r="E24" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B25" t="str">
+        <v>396</v>
+      </c>
+      <c r="C25" t="str">
+        <v>433</v>
+      </c>
+      <c r="D25" t="str" xml:space="preserve">
+        <v xml:space="preserve">اضافة عدد (٣٨) حصة اثرائي لغة انجليزية + (١٢) اثرائي رقمية صفوف أولية فيصبح مجموع الحصص الاثرائية (٥٠) حصة _x000d_
+تخفيض (١) حصة فنية الصف الاول باجمالي (٢) حصة_x000d_
+تخفيض (١) حصة بدنية الصف الاول باجمالي (٢) حصة_x000d_
+تخفيض (١) حصة اسلاميات الصف الاول باجمالي (٢) حصة_x000d_
+تخفيض (١) حصة اسلاميات صفوف عليا باجمالي (٧) حصص_x000d_
+تخفيض حصة رقمية صف 1_x000d_
+استبدال  (٣٢) حصة نشاط  مع الحصص الاثرائية _x000d_
+(٥٠) - (٣٢) = (١٨) حصة </v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v>اسنادات متوسط (بنين)</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v/>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B29" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C29" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+      <c r="D29" t="str">
+        <v>الإسناد</v>
+      </c>
+      <c r="E29" t="str">
+        <v>إجمالي نصاب المعلم</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>فواز المطيري</v>
+      </c>
+      <c r="B30" t="str">
+        <v>اسلاميات</v>
+      </c>
+      <c r="C30" t="str">
+        <v>25</v>
+      </c>
+      <c r="D30" t="str">
+        <v xml:space="preserve"> (5) اسلاميات ص1 فصل 1/1 +(10) اسلاميات ص2 فصلين 2/1 - 2/2 + (10) اسلاميات ص 3 فصل 3/1 - 3/2 </v>
+      </c>
+      <c r="E30" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>احمد صوفي</v>
+      </c>
+      <c r="B31" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C31" t="str">
+        <v>26</v>
+      </c>
+      <c r="D31" t="str">
+        <v xml:space="preserve"> (15) لغتي ص1 متوسط   +  (٥) اسلاميات ص2  فصل 2/3  +(6) تفكير ناقد متوسط ص٣</v>
+      </c>
+      <c r="E31" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>محمد سمير</v>
+      </c>
+      <c r="B32" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C32" t="str">
+        <v>27</v>
+      </c>
+      <c r="D32" t="str">
+        <v xml:space="preserve">(15) لغتي ص2 م + (12 ) لغتي ص 3 </v>
+      </c>
+      <c r="E32" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>ماهر الحربي</v>
+      </c>
+      <c r="B33" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C33" t="str">
+        <v>24</v>
+      </c>
+      <c r="D33" t="str">
+        <v>(18) رياضيات ص١+ (6) رياضيات ص2م فصل 2/3</v>
+      </c>
+      <c r="E33" t="str">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>حسن السيد</v>
+      </c>
+      <c r="B34" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C34" t="str">
+        <v>30</v>
+      </c>
+      <c r="D34" t="str">
+        <v>(18) رياضيات ص3م  + (6) رياضيات ص2م فصل 2/2 - 2/3</v>
+      </c>
+      <c r="E34" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">سلمان الصادق </v>
+      </c>
+      <c r="B35" t="str">
+        <v>لغة انجليزية</v>
+      </c>
+      <c r="C35" t="str">
+        <v>24</v>
+      </c>
+      <c r="D35" t="str">
+        <v xml:space="preserve">(12) انجليزي ص٢متوسط +(12) انجليزي ص٣ متوسط  </v>
+      </c>
+      <c r="E35" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>مصطفى فتحي</v>
+      </c>
+      <c r="B36" t="str">
+        <v>لغة انجليزية</v>
+      </c>
+      <c r="C36" t="str">
+        <v>12</v>
+      </c>
+      <c r="D36" t="str">
+        <v xml:space="preserve"> (١٢) انجليزي ص١ متوسط + مكمل (١٢) حصة بالثانوي </v>
+      </c>
+      <c r="E36" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>فارس الجندي</v>
+      </c>
+      <c r="B37" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C37" t="str">
+        <v>24</v>
+      </c>
+      <c r="D37" t="str">
+        <v xml:space="preserve">(12) علوم ص١ +(12) علوم ص٢ </v>
+      </c>
+      <c r="E37" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">محمد العشماوي </v>
+      </c>
+      <c r="B38" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C38" t="str">
+        <v>27</v>
+      </c>
+      <c r="D38" t="str">
+        <v>(12) علوم ص٣ +(10) اسلاميات ص1 فصل 1/2 - 1/3 + ( 5 ) اسلاميات  صف 3 فصل 3/3</v>
+      </c>
+      <c r="E38" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>عبدالعزيز الربيعان</v>
+      </c>
+      <c r="B39" t="str">
+        <v>اجتماعيات</v>
+      </c>
+      <c r="C39" t="str">
+        <v>24</v>
+      </c>
+      <c r="D39" t="str">
+        <v xml:space="preserve">(24) اجتماعيات (9) ص١ + (9 ) ص٢ +( 6 ) ص٣ متوسط   </v>
+      </c>
+      <c r="E39" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>محمود صابر</v>
+      </c>
+      <c r="B40" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C40" t="str">
+        <v>27</v>
+      </c>
+      <c r="D40" t="str">
+        <v xml:space="preserve">(18) فنية ص١ ص٢ ص٣ + (9) حياتية ص١ + ص2 + ص3 فصل </v>
+      </c>
+      <c r="E40" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>حسين عويضة (مكمل مكرر من الثانوي)</v>
+      </c>
+      <c r="B41" t="str">
+        <v>بدنية</v>
+      </c>
+      <c r="C41" t="str">
+        <v>12</v>
+      </c>
+      <c r="D41" t="str">
+        <v>( 6) بدنية ص2 متوسط +  (6) بدنية ص٣ متوسط + مكمل (١٣) حصة بالثانوي</v>
+      </c>
+      <c r="E41" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>محمد عبد الله (مكمل مكرر من الثانوي)</v>
+      </c>
+      <c r="B42" t="str">
+        <v>رقمية</v>
+      </c>
+      <c r="C42" t="str">
+        <v>8</v>
+      </c>
+      <c r="D42" t="str">
+        <v>(6) رقمية  ص٣ متوسط+ (2) رقمية  ص٢ متوسط فصل 3 + مكمل (١٨) حصة بالثانوي</v>
+      </c>
+      <c r="E42" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">محمود جمعه </v>
+      </c>
+      <c r="B43" t="str">
+        <v>رقمية</v>
+      </c>
+      <c r="C43" t="str">
+        <v>25</v>
+      </c>
+      <c r="D43" t="str">
+        <v>(٦) رقمية  ص١متوسط +(4) رقمية  ص٢ متوسط فصل 1  + فصل 2  + ( 6) بدنية ص1 متوسط + (3) نشاط ص1 + (3) نشاط ص 3 + (3) نشاط ص2</v>
+      </c>
+      <c r="E43" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v>315</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+      <c r="B46" t="str">
+        <v>اسنادات ثانوي (بنين)</v>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v/>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B48" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C48" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+      <c r="D48" t="str">
+        <v>الإسناد</v>
+      </c>
+      <c r="E48" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>احمد نصر</v>
+      </c>
+      <c r="B49" t="str">
+        <v xml:space="preserve">لغة عربية </v>
+      </c>
+      <c r="C49" t="str">
+        <v>24</v>
+      </c>
+      <c r="D49" t="str">
+        <v>20 كفايات 1ث من 6:2 +4 كفايات 2ث 7</v>
+      </c>
+      <c r="E49" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v xml:space="preserve">هشام رسمي </v>
+      </c>
+      <c r="B50" t="str">
+        <v xml:space="preserve">لغة عربية </v>
+      </c>
+      <c r="C50" t="str">
+        <v>27</v>
+      </c>
+      <c r="D50" t="str">
+        <v xml:space="preserve">24 حصة كفايات  2ث 6فصول من 6:1+ 3 حصص 2-ث نون </v>
+      </c>
+      <c r="E50" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v xml:space="preserve">حسن الخطيب </v>
+      </c>
+      <c r="B51" t="str">
+        <v xml:space="preserve">لغة عربية </v>
+      </c>
+      <c r="C51" t="str">
+        <v>24</v>
+      </c>
+      <c r="D51" t="str">
+        <v>14 مهارا ت بحث 3 ث كامل + 6 كفايات 1ث نون  +4 كفايات 1ث 1</v>
+      </c>
+      <c r="E51" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v xml:space="preserve">عبد العزيز الربيعان </v>
+      </c>
+      <c r="B52" t="str">
+        <v xml:space="preserve">لغة عربية </v>
+      </c>
+      <c r="C52" t="str">
+        <v>26</v>
+      </c>
+      <c r="D52" t="str">
+        <v>21 تاريخ 2ث كامل+2 تاريخ 2ث نون +3 تفسير 1ث2 نون</v>
+      </c>
+      <c r="E52" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>خالد المطيري</v>
+      </c>
+      <c r="B53" t="str">
+        <v xml:space="preserve">اسلاميات </v>
+      </c>
+      <c r="C53" t="str">
+        <v>27</v>
+      </c>
+      <c r="D53" t="str">
+        <v xml:space="preserve">24 تفسير وقران 1ث كامل + 3 تفسير 1ث1 نون </v>
+      </c>
+      <c r="E53" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v xml:space="preserve">حسام السيد </v>
+      </c>
+      <c r="B54" t="str">
+        <v xml:space="preserve">رياضيات </v>
+      </c>
+      <c r="C54" t="str">
+        <v>28</v>
+      </c>
+      <c r="D54" t="str">
+        <v xml:space="preserve">20 صف2ث 4 فصول 4:1+4 نون صف2ث + 4 صف3ث1 </v>
+      </c>
+      <c r="E54" t="str">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v xml:space="preserve">محمد سليم </v>
+      </c>
+      <c r="B55" t="str">
+        <v xml:space="preserve">رياضيات </v>
+      </c>
+      <c r="C55" t="str">
+        <v>28</v>
+      </c>
+      <c r="D55" t="str">
+        <v>20صف 3ث من 6:2 +8 حصص 1 ث نون 1-2</v>
+      </c>
+      <c r="E55" t="str">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v xml:space="preserve">وليد الصدة </v>
+      </c>
+      <c r="B56" t="str">
+        <v xml:space="preserve">رياضيات </v>
+      </c>
+      <c r="C56" t="str">
+        <v>24</v>
+      </c>
+      <c r="D56" t="str">
+        <v xml:space="preserve">20 1ث  4 فصول من4:1+ 4 حصص 3ث7 </v>
+      </c>
+      <c r="E56" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>وسيم عبد ربه</v>
+      </c>
+      <c r="B57" t="str">
+        <v xml:space="preserve">رياضيات </v>
+      </c>
+      <c r="C57" t="str">
+        <v>25</v>
+      </c>
+      <c r="D57" t="str">
+        <v>10 صف 1ث  6:5+ 15 صف 2ث من 7:5</v>
+      </c>
+      <c r="E57" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v xml:space="preserve">أحمد طاهر بهيدي </v>
+      </c>
+      <c r="B58" t="str">
+        <v xml:space="preserve">كيمياء </v>
+      </c>
+      <c r="C58" t="str">
+        <v>27</v>
+      </c>
+      <c r="D58" t="str">
+        <v>18 صف 1ث كامل + 6 حصص 1 ث نون 2:1 + 3 علم أرض 3ث7</v>
+      </c>
+      <c r="E58" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v xml:space="preserve">أحمد محمد مصباح </v>
+      </c>
+      <c r="B59" t="str">
+        <v xml:space="preserve">كيمياء </v>
+      </c>
+      <c r="C59" t="str">
+        <v>25</v>
+      </c>
+      <c r="D59" t="str">
+        <v>25 حصة صف2 ث من 5:1</v>
+      </c>
+      <c r="E59" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>محمد متولي</v>
+      </c>
+      <c r="B60" t="str">
+        <v xml:space="preserve">كيمياء </v>
+      </c>
+      <c r="C60" t="str">
+        <v>26</v>
+      </c>
+      <c r="D60" t="str">
+        <v>21 صف 3 ث كامل + 5 حصص 2 ث نون</v>
+      </c>
+      <c r="E60" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>حسن جوده</v>
+      </c>
+      <c r="B61" t="str">
+        <v>كيمياء - فيزياء</v>
+      </c>
+      <c r="C61" t="str">
+        <v>25</v>
+      </c>
+      <c r="D61" t="str">
+        <v>10كيمياء  صف 2ث 7:6+15فيزياء  صف 3ث 3:1</v>
+      </c>
+      <c r="E61" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>فريج السعيد</v>
+      </c>
+      <c r="B62" t="str">
+        <v xml:space="preserve">فيزياء </v>
+      </c>
+      <c r="C62" t="str">
+        <v>24</v>
+      </c>
+      <c r="D62" t="str">
+        <v xml:space="preserve"> 20صف 3ث 7:4 + 4 حصص 2 ث7</v>
+      </c>
+      <c r="E62" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v xml:space="preserve">سلمان محمد </v>
+      </c>
+      <c r="B63" t="str">
+        <v xml:space="preserve">فيزياء </v>
+      </c>
+      <c r="C63" t="str">
+        <v>28</v>
+      </c>
+      <c r="D63" t="str">
+        <v xml:space="preserve">24 حصة صف2 ث 6 فصول 6:1 + 4 حصص 2ث نون </v>
+      </c>
+      <c r="E63" t="str">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v xml:space="preserve">محمد عبد المنعم </v>
+      </c>
+      <c r="B64" t="str">
+        <v xml:space="preserve">أحياء </v>
+      </c>
+      <c r="C64" t="str">
+        <v>27</v>
+      </c>
+      <c r="D64" t="str">
+        <v>18 صف 1ث كامل + 3 علم ارض ص ثالث6 +6 حصص 1 ث نون 1و2</v>
+      </c>
+      <c r="E64" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>حسن ابوغنيمة</v>
+      </c>
+      <c r="B65" t="str">
+        <v xml:space="preserve">أحياء </v>
+      </c>
+      <c r="C65" t="str">
+        <v>20</v>
+      </c>
+      <c r="D65" t="str">
+        <v>20 حصة 2ث 4:1+4أحياء  2ث نون+ مسند له كلاسيرا</v>
+      </c>
+      <c r="E65" t="str">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>محمد علي</v>
+      </c>
+      <c r="B66" t="str">
+        <v xml:space="preserve">أحياء </v>
+      </c>
+      <c r="C66" t="str">
+        <v>27</v>
+      </c>
+      <c r="D66" t="str">
+        <v>15 علم أرض 3ث من 5:3 + 12 أحياءص2ث 7:5</v>
+      </c>
+      <c r="E66" t="str">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v xml:space="preserve">مصطفى محمد </v>
+      </c>
+      <c r="B67" t="str">
+        <v xml:space="preserve">لغة انجليزية </v>
+      </c>
+      <c r="C67" t="str">
+        <v>26</v>
+      </c>
+      <c r="D67" t="str">
+        <v>24حصة اث كامل + 2 حصة 1ث نون 1</v>
+      </c>
+      <c r="E67" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v xml:space="preserve">عبد الرحمن شطا </v>
+      </c>
+      <c r="B68" t="str">
+        <v xml:space="preserve">لغة انجليزية </v>
+      </c>
+      <c r="C68" t="str">
+        <v>25</v>
+      </c>
+      <c r="D68" t="str">
+        <v>20حصة 2 ث من5:1+ 4 حصص 3ث1+ 1 حصة نون 2ث</v>
+      </c>
+      <c r="E68" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v xml:space="preserve">مصطفى فتحي (مكرر مكمل من المتوسط) </v>
+      </c>
+      <c r="B69" t="str">
+        <v xml:space="preserve">لغة انجليزية </v>
+      </c>
+      <c r="C69" t="str">
+        <v>12</v>
+      </c>
+      <c r="D69" t="str">
+        <v>8 حصص 2 ث 6 و7 + 4 تفكير ناقد صف 1ث نون 1و2 + مكمل (١٢) حصة بالمتوسط</v>
+      </c>
+      <c r="E69" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>إبراهيم شبكة</v>
+      </c>
+      <c r="B70" t="str">
+        <v xml:space="preserve">لغة انجليزية </v>
+      </c>
+      <c r="C70" t="str">
+        <v>24</v>
+      </c>
+      <c r="D70" t="str">
+        <v>24 حصة صف 3ث 7:2</v>
+      </c>
+      <c r="E70" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>احمد توفيق</v>
+      </c>
+      <c r="B71" t="str">
+        <v>تقنية -حاسب</v>
+      </c>
+      <c r="C71" t="str">
+        <v>24</v>
+      </c>
+      <c r="D71" t="str">
+        <v>20 حصة مجال صف 3 ث 5:1+ 4 حصص 1ث نون تقنية 1و2</v>
+      </c>
+      <c r="E71" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v xml:space="preserve">محمد مدحت </v>
+      </c>
+      <c r="B72" t="str">
+        <v>تقنية -حاسب</v>
+      </c>
+      <c r="C72" t="str">
+        <v>24</v>
+      </c>
+      <c r="D72" t="str">
+        <v xml:space="preserve">18 حصة 1ث كامل  + 6تفكير ناقد 1ث </v>
+      </c>
+      <c r="E72" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v xml:space="preserve">محمد صلاح </v>
+      </c>
+      <c r="B73" t="str">
+        <v xml:space="preserve">بدنية </v>
+      </c>
+      <c r="C73" t="str">
+        <v>28</v>
+      </c>
+      <c r="D73" t="str">
+        <v>12حصة 1ث كامل+12بدنية 3ث من  4:1 + 4 صف اول نون 1و2</v>
+      </c>
+      <c r="E73" t="str">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v xml:space="preserve">حسين عويضة </v>
+      </c>
+      <c r="B74" t="str">
+        <v xml:space="preserve">بدنية </v>
+      </c>
+      <c r="C74" t="str">
+        <v>13</v>
+      </c>
+      <c r="D74" t="str">
+        <v>9بدنية 3ث 7:5 + 8 مجال اختياري 3ث6 (م بالمتوسط بعد الفسحة) + مكمل (١٢) حصة بالمتوسط</v>
+      </c>
+      <c r="E74" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v xml:space="preserve">عيد العتيبي + (م .اداري)   </v>
+      </c>
+      <c r="B75" t="str">
+        <v xml:space="preserve">علم نفس </v>
+      </c>
+      <c r="C75" t="str">
+        <v>13</v>
+      </c>
+      <c r="D75" t="str">
+        <v xml:space="preserve"> 6 تفكير ناقد 1ث+ 7 نشاط 2ث + مكمل مراقب دور</v>
+      </c>
+      <c r="E75" t="str">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>محمد عبد الله</v>
+      </c>
+      <c r="B76" t="str">
+        <v>تقنية -حاسب</v>
+      </c>
+      <c r="C76" t="str">
+        <v>18</v>
+      </c>
+      <c r="D76" t="str">
+        <v>14 تقنية 3ث كامل + 4 مجال صف 3 ث 7+ مكمل (٨) حصص بالمتوسط</v>
+      </c>
+      <c r="E76" t="str">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="77" xml:space="preserve">
+      <c r="A77" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B77" t="str">
+        <v/>
+      </c>
+      <c r="C77" t="str">
+        <v/>
+      </c>
+      <c r="D77" t="str" xml:space="preserve">
+        <v xml:space="preserve">تخفيض حصة من اللغة الإنجليزية أول ثانوي_x000d_
+تخفيض حصة من اللغة الإنجليزيةوثان _x000d_
+تخفيض حصة تفكير ناقد أول ثانوي _x000d_
+تخفيض حصة نشاط صف ثان ثانوي_x000d_
+تخفيض حصة نشاط صف ثالث ثانوي _x000d_
+تخفيض حصة مجال صف ثالث ثانوي _x000d_
+عليه خروج جميع طلاب المدرسة بعد الحصة السادسة يوميا 11:50( بواقع تخفيض حصتين من كل فصل ) </v>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v/>
+      </c>
+      <c r="B78" t="str">
+        <v/>
+      </c>
+      <c r="C78" t="str">
+        <v/>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v/>
+      </c>
+      <c r="B79" t="str">
+        <v>========================================</v>
+      </c>
+      <c r="C79" t="str">
+        <v/>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v>اسنادات قطاع البنات</v>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v/>
+      </c>
+      <c r="B81" t="str">
+        <v/>
+      </c>
+      <c r="C81" t="str">
+        <v/>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v/>
+      </c>
+      <c r="B82" t="str">
+        <v>اسنادات ابتدائي (بنات)</v>
+      </c>
+      <c r="C82" t="str">
+        <v/>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B83" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C83" t="str">
+        <v xml:space="preserve">عدد حصص المعلم بالمرحلة </v>
+      </c>
+      <c r="D83" t="str">
+        <v>ملاحظات</v>
+      </c>
+      <c r="E83" t="str">
+        <v>إجمالي نصاب المعلم بعد الاكمال</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v/>
+      </c>
+      <c r="B84" t="str">
+        <v/>
+      </c>
+      <c r="C84" t="str">
+        <v/>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v xml:space="preserve">نورا مجدي </v>
+      </c>
+      <c r="B85" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C85">
+        <v>24</v>
+      </c>
+      <c r="D85" t="str">
+        <v>(3) انجليزي وزاري ص1 ( 2) انجليزي اثرائي ص1 (1) ماث ص1 ( 1) ساينس ص1 ( 3) انجليزي وزاري ص2 (2) انجليزي اثرائي ص2 (6) انجليزي وزاري ص3 (4)انجليزي اثرائي ص3 (2) نشاط ص5</v>
+      </c>
+      <c r="E85">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v xml:space="preserve">سارة المخلفي </v>
+      </c>
+      <c r="B86" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C86">
+        <v>24</v>
+      </c>
+      <c r="D86" t="str">
+        <v>(10)اسلاميةص3(5)اسلاميةص4(5)إسلامية ص5(2)اجتماعيات ص5(2)نشاط ص4 + منسقة تطوع ابتدائي ومتوسط</v>
+      </c>
+      <c r="E86">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>نوير الشمري ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B87" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C87">
+        <v>8</v>
+      </c>
+      <c r="D87" t="str">
+        <v>(2) رقمية ص2 (2)رقمية ص4(2)رقمية ص5(2) رقمية ص6 + مسند (٦) حصص بالمتوسط + (10) حصة بالثانوي</v>
+      </c>
+      <c r="E87">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>نهال الشبرمي ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B88" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C88">
+        <v>7</v>
+      </c>
+      <c r="D88" t="str">
+        <v>(2) بدنية ص6 (5) إسلامية ص6 + مسند (13) حصة بالمتوسط + (4) رقمية kg + منسقة الصيانة والمشتريات</v>
+      </c>
+      <c r="E88">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v xml:space="preserve">نوضا المطيري </v>
+      </c>
+      <c r="B89" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C89">
+        <v>24</v>
+      </c>
+      <c r="D89" t="str">
+        <v>(4)رياضيات ص1(3) علوم ص1 (3) علوم ص2 (6) رياضيات ص4 (2)اجتماعايت ص4 (1) اسرية ص4(1) نشاط ص3 فصل(4) رقمية ص3</v>
+      </c>
+      <c r="E89">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>الجوهرة المخلفي  ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B90" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C90">
+        <v>7</v>
+      </c>
+      <c r="D90" t="str">
+        <v>(5) لغتي ص6 (2) اجتماعيات ص6 + (17) حصة بالمتوسط + منسقة اختبارات مركزية</v>
+      </c>
+      <c r="E90">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>حنان العنزي (مكرر مكمل من متوسط )</v>
+      </c>
+      <c r="B91" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91" t="str">
+        <v>(3) بدنية ص1 + مسند لها ( 11 ) متوسط + (11) ثانوي + منسقة اختبارات steep</v>
+      </c>
+      <c r="E91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>أشواق العنزي</v>
+      </c>
+      <c r="B92" t="str">
+        <v xml:space="preserve"> لغة عربية</v>
+      </c>
+      <c r="C92">
+        <v>25</v>
+      </c>
+      <c r="D92" t="str">
+        <v>(8)لغتي ص1 (7)لغتي ص2 (5) إسلامية ص1(5) إسلامية ص2</v>
+      </c>
+      <c r="E92">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>ناهد بعزقي</v>
+      </c>
+      <c r="B93" t="str">
+        <v xml:space="preserve"> لغة عربية</v>
+      </c>
+      <c r="C93">
+        <v>24</v>
+      </c>
+      <c r="D93" t="str">
+        <v>(12) لغتي ص3 (5)لغتي ص4 (5) لغتي ص5 (1)اسرية ص5 (1) نشاط ص 3فصل</v>
+      </c>
+      <c r="E93">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>نوف الزلفي</v>
+      </c>
+      <c r="B94" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C94">
+        <v>24</v>
+      </c>
+      <c r="D94" t="str">
+        <v>(6)رياضيات ص2 (12) رياضيات ص3 (6) بدنية ص3 + معلمة موهبة</v>
+      </c>
+      <c r="E94">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>نور العيدة ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B95" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C95">
+        <v>6</v>
+      </c>
+      <c r="D95" t="str">
+        <v xml:space="preserve"> ( 6 )  رياضيات ص6 + مسند ( 18) ثانوي + منسقة قدرات وتحصيلي</v>
+      </c>
+      <c r="E95">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>هدى المطيري ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B96" t="str">
+        <v>كيمياء</v>
+      </c>
+      <c r="C96">
+        <v>2</v>
+      </c>
+      <c r="D96" t="str">
+        <v>(2) بدنية ص5 + مسند ( 23) ثانوي</v>
+      </c>
+      <c r="E96">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>سلطانة العتيبي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B97" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C97">
+        <v>1</v>
+      </c>
+      <c r="D97" t="str">
+        <v>(1) اسرية ص6 + ( 18 ) ثانوي + ( 5) متوسط</v>
+      </c>
+      <c r="E97">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>نوف العتيبي ( مكرر مكمل من الثانوي )</v>
+      </c>
+      <c r="B98" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C98">
+        <v>2</v>
+      </c>
+      <c r="D98" t="str">
+        <v>(2) رقمية ص1 + (22) مسند ثانوي</v>
+      </c>
+      <c r="E98">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>بدور  البقمي  ( مكرر مكمل من المتوسط)</v>
+      </c>
+      <c r="B99" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C99">
+        <v>6</v>
+      </c>
+      <c r="D99" t="str">
+        <v>(6)رياضيات ص5 + مسند ( 18)  متوسط</v>
+      </c>
+      <c r="E99">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>منى الخلف</v>
+      </c>
+      <c r="B100" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C100">
+        <v>20</v>
+      </c>
+      <c r="D100" t="str">
+        <v xml:space="preserve"> (8) علوم ص3 (4) علوم ص4 (4) علوم ص5  (4) علوم ص6 + مسند (4) بالمتوسط</v>
+      </c>
+      <c r="E100">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v xml:space="preserve"> عهود الرويلي </v>
+      </c>
+      <c r="B101" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C101">
+        <v>20</v>
+      </c>
+      <c r="D101" t="str">
+        <v>(3) انجليزي وزاري ص4 ( 2) انجليزي اثرائي ص4  ( 3) انجليزي وزاري ص5 (2) انجليزي اثرائي ص5 (3) انجليزي وزاري ص6 (2)انجليزي اثرائي ص6 (3) بدنية ص2 (2) نشاط ص6 + (4) kg</v>
+      </c>
+      <c r="E101">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v xml:space="preserve">هدى البكري </v>
+      </c>
+      <c r="B102" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C102">
+        <v>18</v>
+      </c>
+      <c r="D102" t="str">
+        <v>(2)فنية ص1(2) فنية ص2(4) فنية ص3(1) فنية ص4(1)فنية ص5(1) قنية ص6  (2) بدنية ص4 (1)نشاط ص2 (1) اسرية ص1(1) اسرية ص2(2)اسرية ص3+ مسند (6) حصص بالمتوسط + موجهة صحية ابتدائي</v>
+      </c>
+      <c r="E102">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B103">
+        <v>245</v>
+      </c>
+      <c r="C103">
+        <v>245</v>
+      </c>
+      <c r="D103" t="str">
+        <v>تم زيادة ( 14) حصة لتفعيل المواد الاثرائية ورفع مستوى التحصيل فأصبح إجمالي الحصص في الأسبوع 35</v>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v/>
+      </c>
+      <c r="B104" t="str">
+        <v>اسنادات متوسط (بنات)</v>
+      </c>
+      <c r="C104" t="str">
+        <v/>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B105" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C105" t="str">
+        <v xml:space="preserve">عدد حصص المعلم بالمرحلة </v>
+      </c>
+      <c r="D105" t="str">
+        <v>ملاحظات</v>
+      </c>
+      <c r="E105" t="str">
+        <v>إجمالي نصاب المعلم بعد الاكمال</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v/>
+      </c>
+      <c r="B106" t="str">
+        <v/>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>هدى البكري ( مكرر مكمل من ابتدائي)</v>
+      </c>
+      <c r="B107" t="str">
+        <v>فنية</v>
+      </c>
+      <c r="C107">
+        <v>6</v>
+      </c>
+      <c r="D107" t="str">
+        <v>(2) فنية ص1 (2) فنية ص2 (2) فنية ص + مسند (18) حصة بالابتدائي + موجهة صحية ابتدائي</v>
+      </c>
+      <c r="E107">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v xml:space="preserve">حنان الغربي </v>
+      </c>
+      <c r="B108" t="str">
+        <v>اجتماعيات</v>
+      </c>
+      <c r="C108">
+        <v>11</v>
+      </c>
+      <c r="D108" t="str">
+        <v>(3) اجتماعيات ص1 (3) اجتماعيات ص2(2) اجتماعيات ص3 (2) بدنية 3م (1) اسرية 3م + مسند (13) حصص بالثانوي + مسؤولة المقصف</v>
+      </c>
+      <c r="E108">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>نوير الشمري    ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B109" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C109">
+        <v>6</v>
+      </c>
+      <c r="D109" t="str">
+        <v>(2) رقمية ص1 (2) رقمية ص3 (2) رقمية ص3 + مسند (١0) حصص بالثانوي + (8) حصص بالابتدائي</v>
+      </c>
+      <c r="E109">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>منى الخلف ( مكرر مكمل من الابتدائي )</v>
+      </c>
+      <c r="B110" t="str">
+        <v>علوم</v>
+      </c>
+      <c r="C110">
+        <v>4</v>
+      </c>
+      <c r="D110" t="str">
+        <v>(4) علوم ص1 + مسند (20 ) ابتدائي</v>
+      </c>
+      <c r="E110">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>بدور  البقمي</v>
+      </c>
+      <c r="B111" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C111">
+        <v>18</v>
+      </c>
+      <c r="D111" t="str">
+        <v>(6) رياضيات ص1 (6) رياضيات ص2 (6) رياضيات ص3 + مسند لها (6) ابتدائي</v>
+      </c>
+      <c r="E111">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>ريم الحربي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B112" t="str">
+        <v>دين</v>
+      </c>
+      <c r="C112">
+        <v>5</v>
+      </c>
+      <c r="D112" t="str">
+        <v>( 5 ) إسلامية ص3 + مسند ثانوي 19 ثانوي</v>
+      </c>
+      <c r="E112">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>اماني فهمي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B113" t="str">
+        <v>احياء</v>
+      </c>
+      <c r="C113">
+        <v>4</v>
+      </c>
+      <c r="D113" t="str">
+        <v>(4) علوم ص2 + مسند لها (20) ثانوي</v>
+      </c>
+      <c r="E113">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>سلطانة العتيبي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B114" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C114">
+        <v>5</v>
+      </c>
+      <c r="D114" t="str">
+        <v>(4) علوم ص3 (1) نشاط ص3 + مسند لها (18 ) ثانوي + ( 1) ابتدائي + منسقة نافس</v>
+      </c>
+      <c r="E114">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>امل العنزي ( مكرر مكمل من الثانوي)</v>
+      </c>
+      <c r="B115" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C115">
+        <v>5</v>
+      </c>
+      <c r="D115" t="str">
+        <v>(4) انجليزي ص3 (1) أسرية ص3 + مسند (19) حصة بالثانوي + منسقة اختبارات steep</v>
+      </c>
+      <c r="E115">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>حنان العنزي</v>
+      </c>
+      <c r="B116" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C116">
+        <v>11</v>
+      </c>
+      <c r="D116" t="str">
+        <v>(4) انجليزي ص1(4) انجليزي ص2(1)اسرية ص2 (2) بدنية ص2+ مسند لها (11) حصة ثانوي+(3) ابتدائي</v>
+      </c>
+      <c r="E116">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>الجوهرة المخلفي</v>
+      </c>
+      <c r="B117" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C117">
+        <v>17</v>
+      </c>
+      <c r="D117" t="str">
+        <v>(5) لغتي ص1 (5) لغتي ص2(4) لغتي ص3 (2) بدنية ص1 (1) نشاط ص1 + مسند (7) حصص بالابتدائي + منسقة اختبارات مركزية</v>
+      </c>
+      <c r="E117">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>نهال الشبرمي</v>
+      </c>
+      <c r="B118" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C118">
+        <v>13</v>
+      </c>
+      <c r="D118" t="str">
+        <v>(5) إسلامية ص1 (5) إسلامية ص2  (٢)  تفكير ناقد ص3  (1) نشاط ص2 + مسند (7) حصص بالابتدائي + (4) kg + منسقة الصيانة والمشتريات</v>
+      </c>
+      <c r="E118">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B119">
+        <v>105</v>
+      </c>
+      <c r="C119">
+        <v>105</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v/>
+      </c>
+      <c r="B120" t="str">
+        <v>اسنادات ثانوي (بنات)</v>
+      </c>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>المعلم</v>
+      </c>
+      <c r="B121" t="str">
+        <v>المادة</v>
+      </c>
+      <c r="C121" t="str">
+        <v>عدد حصص المعلم بالمدرسة</v>
+      </c>
+      <c r="D121" t="str">
+        <v>الإسناد</v>
+      </c>
+      <c r="E121" t="str">
+        <v>إجمالي نصاب المعلم</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>حنان الغربي ( مكرر مكمل  متوسط )</v>
+      </c>
+      <c r="B122" t="str">
+        <v>اجتماعيات</v>
+      </c>
+      <c r="C122">
+        <v>13</v>
+      </c>
+      <c r="D122" t="str">
+        <v>(6) تاريخ ص2 (6) بدنية ص3 (1) نشاط ص3 فصل + مسند (11) حصص بالمتوسط + مسؤولة المقصف</v>
+      </c>
+      <c r="E122">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v xml:space="preserve">نوف العتيبي </v>
+      </c>
+      <c r="B123" t="str">
+        <v>لغة عربية</v>
+      </c>
+      <c r="C123">
+        <v>22</v>
+      </c>
+      <c r="D123" t="str">
+        <v>(8) كفايات ص1(8) كفايات ص2 (4) بحث ومعلومات ص3 (2) نشاط ص2  + مسند (2) ابتدائي + أمينة مصادر</v>
+      </c>
+      <c r="E123">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>ريم الحربي</v>
+      </c>
+      <c r="B124" t="str">
+        <v>إسلامية</v>
+      </c>
+      <c r="C124">
+        <v>19</v>
+      </c>
+      <c r="D124" t="str">
+        <v>(6) تفكير ناقد ص1 (8) قرآن وتفسيره صف1 (5) مجال اختياري مهارات إدارية + مسند (5) متوسط</v>
+      </c>
+      <c r="E124">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>سلطانة البقمي</v>
+      </c>
+      <c r="B125" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C125">
+        <v>25</v>
+      </c>
+      <c r="D125" t="str">
+        <v xml:space="preserve">(8) رياضيات ص3 (10) رياضيات ص1 ( 4) بدنية ص1 (3) نشاط ص3 </v>
+      </c>
+      <c r="E125">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>نور العيدة</v>
+      </c>
+      <c r="B126" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="C126">
+        <v>18</v>
+      </c>
+      <c r="D126" t="str">
+        <v>(10) رياضيات ص2 (3) نشاط ص2 (5) مجال اختياري تنمية مستدامة ص3 + مسند (6) ابتدائي+ منسقة قدرات وتحصيلي</v>
+      </c>
+      <c r="E126">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>سلطانة العتيبي</v>
+      </c>
+      <c r="B127" t="str">
+        <v>فيزياء</v>
+      </c>
+      <c r="C127">
+        <v>18</v>
+      </c>
+      <c r="D127" t="str">
+        <v>(8) فيزياء ص2 (10) فيزياء ص3 + مسند (5) متوسط + (1) ابتدائي  + منسقة نافس</v>
+      </c>
+      <c r="E127">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>هدى المطيري</v>
+      </c>
+      <c r="B128" t="str">
+        <v>كيمياء</v>
+      </c>
+      <c r="C128">
+        <v>23</v>
+      </c>
+      <c r="D128" t="str">
+        <v>(6) كيمياء ص1 (10) كيمياء ص2 (6) كيمياء ص3 (1) نشاط ص1 فصل + (2) مسند ابتدائي</v>
+      </c>
+      <c r="E128">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>أماني فهمي</v>
+      </c>
+      <c r="B129" t="str">
+        <v>أحياء</v>
+      </c>
+      <c r="C129">
+        <v>20</v>
+      </c>
+      <c r="D129" t="str">
+        <v>(6) أحياء ص1 (8) أحياء ص2 (9) علم الأرض ص3 + مسند (4) متوسط</v>
+      </c>
+      <c r="E129">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>حنان العنزي (مكرر مكمل من متوسط )</v>
+      </c>
+      <c r="B130" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C130">
+        <v>11</v>
+      </c>
+      <c r="D130" t="str">
+        <v>(10) انجليزي ص1 (1) نشاط ص1 فصل + مسند (11) متوسط +( 3) ابتدائي</v>
+      </c>
+      <c r="E130">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v xml:space="preserve">أمل العنزي </v>
+      </c>
+      <c r="B131" t="str">
+        <v>انجليزي</v>
+      </c>
+      <c r="C131">
+        <v>19</v>
+      </c>
+      <c r="D131" t="str">
+        <v>(8) انجليزي ص3 (10) انجليزي ص2 (1) نشاط ص2 فصل + مسند (5) متوسط + منسقة اختبارات steep</v>
+      </c>
+      <c r="E131">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v xml:space="preserve">نوير الشمري </v>
+      </c>
+      <c r="B132" t="str">
+        <v>حاسب</v>
+      </c>
+      <c r="C132">
+        <v>10</v>
+      </c>
+      <c r="D132" t="str">
+        <v>(٦) تقنية رقمية ص1 (4) رقمية ص3  + مسند (٦) حصص بالمتوسط + (8) حصص بالابتدائي</v>
+      </c>
+      <c r="E132">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>إجمالي الحصص</v>
+      </c>
+      <c r="B133">
+        <v>198</v>
+      </c>
+      <c r="C133">
+        <v>198</v>
+      </c>
+      <c r="D133" t="str">
+        <v>تم زيادة ( 6) حصص لتفعيل البرامج الاثرائية ورفع مستوى التحصيل فأصبحت إجمالي الحصص 198</v>
+      </c>
+      <c r="E133" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E133"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N59"/>

</xml_diff>